<commit_message>
Update scanner pending logic
</commit_message>
<xml_diff>
--- a/auto-scanner/outputs/자동진단.xlsx
+++ b/auto-scanner/outputs/자동진단.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -445,7 +445,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -552,7 +552,17 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -576,7 +586,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="51" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
@@ -642,7 +652,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -652,7 +662,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -682,24 +692,24 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>anonymous_request 기준으로 비로그인 요청 시 /vulnapp/admin.jsp는 상태코드 302를 반환하고 Location 헤더가 /vulnapp/login.jsp로 설정되어 로그인 페이지로 리다이렉트됨. 관리자 본문 노출 근거가 없어 비로그인 직접 접근은 방어된 것으로 판단함. 단, 로그인 후 일반 사용자 권한으로 관리자 기능 접근 가능 여부는 별도 권한 검증이 필요함. 시그니처 기반 추가 근거: /vulnapp/admin.jsp 비로그인 요청은 로그인 페이지로 리다이렉트됨. 일반 사용자 권한 우회 여부는 인증 계정 기반 추가 진단 필요.</t>
+          <t>익명 요청은 /vulnapp/admin.jsp에서 302로 /vulnapp/login.jsp로 리다이렉트되었으나, 일반 사용자 계정(user1) 로그인 후 동일한 /vulnapp/admin.jsp 요청이 status_code 200으로 응답하였다. 응답 본문에 "⚙️ 시스템 관리자 대시보드", "Admin Only", "현재 서버에 가입된 모든 회원" 문구가 포함되어 일반 사용자가 관리자 전용 페이지에 접근 가능한 것으로 확인된다. 시그니처 기반 추가 근거: /vulnapp/admin.jsp 비로그인 요청은 로그인 페이지로 리다이렉트됨. 일반 사용자(user1) 로그인 세션으로 /vulnapp/admin.jsp 접근 시 200 응답과 관리자 페이지 키워드가 확인되어 관리자 권한 검증 미흡이 확인됨.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>현재 확인된 비로그인 직접 접근 차단은 유지하되, 인증 이후에도 관리자 권한을 서버 측에서 검증하고 일반 사용자 세션의 관리자 페이지 접근을 403 또는 안전한 거부 응답으로 차단하라.</t>
+          <t>관리자 기능은 서버 측에서 사용자 역할/권한을 검증하여 관리자 권한이 없는 세션은 403 처리하거나 접근을 차단해야 한다. 모든 관리자 페이지와 API에 동일한 권한 검사를 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -709,7 +719,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -744,19 +754,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 수집 근거에는 /vulnapp/profile.jsp?user_idx=1 단일 요청의 200 응답만 있어 IDOR 확정이 어려웠으나, 시그니처 기반 보조 근거에서 profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출된 것으로 보고됨. 시그니처 기반 추가 근거: profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출됨.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 시그니처 기반 보조 근거에 따르면 profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출되는 것으로 보고되었다. collected_evidence에는 /vulnapp/profile.jsp?user_idx=1의 200 응답만 있고 사용자 간 비교 본문은 부족하므로, 시그니처 결과를 보조 근거로 최종 취약 판단한다. 시그니처 기반 추가 근거: profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출됨.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>사용자 정보 조회 시 세션 사용자와 조회 대상 user_idx의 소유권을 서버 측에서 검증하고, 권한 없는 객체 접근은 403으로 차단하라. 객체 식별자만 변경해 타 사용자 정보가 조회되지 않도록 접근통제 로직을 중앙화하라.</t>
+          <t>사용자 정보 조회 시 세션 사용자와 조회 대상 객체의 소유자 또는 권한을 서버 측에서 검증하고, 권한 없는 user_idx 접근은 403 또는 일반화된 오류로 차단해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -766,7 +776,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -801,19 +811,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>기본 페이지 응답 헤더에는 Server, Date, Content-Type, Transfer-Encoding, Connection, Content-Encoding만 확인되며 Content-Security-Policy, X-Frame-Options 또는 frame-ancestors, X-Content-Type-Options, Referrer-Policy, Permissions-Policy, Strict-Transport-Security 등 주요 보안 헤더가 확인되지 않음. /vulnapp/search.jsp 응답에서도 유사하게 주요 보안 헤더가 확인되지 않음. 시그니처 기반 추가 근거: /vulnapp/ 응답에서 주요 보안 헤더 누락: ['Content-Security-Policy', 'X-Frame-Options', 'X-Content-Type-Options', 'Referrer-Policy']</t>
+          <t>기본 페이지 http://15.164.60.79/ 응답 헤더에서 Content-Security-Policy, X-Frame-Options 또는 frame-ancestors, X-Content-Type-Options, Referrer-Policy, Strict-Transport-Security 등의 주요 보안 헤더가 확인되지 않는다. 시그니처 기반 추가 근거: /vulnapp/ 응답에서 주요 보안 헤더 누락: ['Content-Security-Policy', 'X-Frame-Options', 'X-Content-Type-Options', 'Referrer-Policy']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Content-Security-Policy, X-Content-Type-Options: nosniff, X-Frame-Options 또는 CSP frame-ancestors, Referrer-Policy, Permissions-Policy를 설정하고, HTTPS 적용 후 Strict-Transport-Security를 활성화하라.</t>
+          <t>Content-Security-Policy, X-Frame-Options 또는 CSP frame-ancestors, X-Content-Type-Options: nosniff, Referrer-Policy, Permissions-Policy 등을 설정한다. HTTPS 적용 후 HSTS도 설정한다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -823,7 +833,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -858,19 +868,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>응답 헤더 Server 값이 "nginx/1.28.3 (Ubuntu)"로 제품명, 버전, OS 정보를 노출함. 기본 페이지 본문 title 및 h1에 "Apache Tomcat/9.0.118"가 표시되고, 404 오류 페이지 하단에도 "Apache Tomcat/9.0.118"가 노출됨. 시그니처 기반 추가 근거: http://15.164.60.79/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79/ body contains Apache Tomcat/; http://15.164.60.79/vulnapp/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79:8080/ body contains Apache Tomcat/</t>
+          <t>http://15.164.60.79/ 응답 헤더에 "Server: nginx/1.28.3 (Ubuntu)"가 노출된다. 또한 기본 페이지 본문 title 및 h1, 404 오류 페이지 하단에 "Apache Tomcat/9.0.118"가 노출된다. 시그니처 기반 추가 근거: http://15.164.60.79/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79/ body contains Apache Tomcat/; http://15.164.60.79/vulnapp/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79:8080/ body contains Apache Tomcat/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>nginx server_tokens를 비활성화하고 프록시 및 애플리케이션 서버의 상세 버전 노출을 최소화하라. Tomcat 기본/오류 페이지를 사용자 정의 페이지로 대체하여 제품명과 상세 버전 문자열을 제거하라.</t>
+          <t>nginx의 server_tokens를 비활성화하고, Tomcat 기본/오류 페이지에서 제품명 및 상세 버전이 노출되지 않도록 커스텀 오류 페이지와 배너 제거 설정을 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -880,7 +890,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -915,19 +925,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>http://15.164.60.79:8080/ 및 http://15.164.60.79/ 이 상태코드 200으로 응답하고 본문에 "Apache Tomcat/9.0.118", "If you're seeing this, you've successfully installed Tomcat. Congratulations!" 및 Documentation, Configuration, Examples 링크가 포함된 Tomcat 기본 페이지가 노출됨. 시그니처 기반 추가 근거: http://15.164.60.79:8080/에서 Tomcat 기본 페이지와 Manager/Host Manager 링크 노출</t>
+          <t>http://15.164.60.79:8080/ 및 http://15.164.60.79/ 요청이 status_code 200으로 응답했고, 본문에 "Apache Tomcat/9.0.118", "If you're seeing this, you've successfully installed Tomcat. Congratulations!", /docs/, /examples/ 링크 등 Tomcat 기본 페이지 내용이 확인된다. 시그니처 기반 추가 근거: http://15.164.60.79:8080/에서 Tomcat 기본 페이지와 Manager/Host Manager 링크 노출</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>운영 환경에서 Tomcat ROOT 기본 애플리케이션, docs, examples 등 기본 리소스를 제거하고 필요한 애플리케이션만 배포하라. 8080 포트의 외부 접근을 제한하고 관리용 포트와 서비스 포트를 분리하라.</t>
+          <t>운영 환경에서는 Tomcat ROOT 기본 애플리케이션, docs, examples 등 불필요한 기본 리소스를 제거하고 실제 서비스 페이지 또는 차단 페이지로 대체한다. 8080 포트의 외부 노출 필요성도 재검토한다.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -937,7 +947,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -967,24 +977,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>/vulnapp/debug.jsp 및 /vulnapp/debug.jsp?debug=true가 상태코드 200으로 응답하며 Content-Type은 application/json;charset=UTF-8임. 본문에 "debug": true, "db_user": "vulnuser", "db_password": "vulnpass1234", "api_key": "TEST-API-KEY-123456", "internal_ip": "10.0.0.5"가 노출됨. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/debug.jsp에서 debug/API 키/DB 계정/내부 IP 등 내부 정보 노출</t>
+          <t>http://15.164.60.79/vulnapp/debug.jsp와 /vulnapp/debug.jsp?debug=true가 모두 status_code 200, Content-Type application/json으로 응답했다. 본문에 "debug": true와 함께 "db_user": "vulnuser", "db_password": "vulnpass1234", "api_key": "TEST-API-KEY-123456", "internal_ip": "10.0.0.5"가 노출된다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/debug.jsp에서 debug/API 키/DB 계정/내부 IP 등 내부 정보 노출</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>운영 환경에서 디버그 엔드포인트를 제거하거나 인증/인가 뒤로 이동하고, DB 계정, 비밀번호, API 키, 내부 IP 등 민감정보를 응답에서 제거하라. 이미 노출된 자격증명은 즉시 폐기 및 재발급하라.</t>
+          <t>운영 환경에서 debug 기능과 debug 엔드포인트를 비활성화하거나 인증/인가된 관리자에게만 제한한다. 노출된 DB 계정 비밀번호와 API 키는 즉시 폐기 및 재발급하고, 민감정보가 응답에 포함되지 않도록 제거한다.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -994,7 +1004,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1029,19 +1039,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 수집된 HTTP 응답과 시그니처 기반 보조 근거 모두 외부 응답에서 Log4j 사용 흔적이나 버전 정보를 확인하지 못함. 서버 내부 의존성 목록이 없어 취약한 Log4j 사용 여부는 판단할 수 없음. 시그니처 기반 추가 근거: 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않음. 서버 내부 라이브러리 확인은 수동진단으로 보완 필요.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 시그니처 기반 보조 근거에서 외부 HTTP 응답상 Log4j 사용 흔적이 확인되지 않았고, collected_evidence에도 Log4j 라이브러리나 취약 버전을 판단할 근거가 없다. 현재 외부 진단 범위에서는 진단 대상 기능 또는 사용 흔적이 확인되지 않아 n/a로 판단한다. 시그니처 기반 추가 근거: 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않음. 서버 내부 라이브러리 확인은 수동진단으로 보완 필요.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>서버 배포물, 빌드 파일, SBOM, 라이브러리 디렉터리에서 Log4j 사용 여부와 버전을 확인하고, 취약 버전이 확인되면 안전한 지원 버전으로 업그레이드하라.</t>
+          <t>서버 내부 SBOM, WEB-INF/lib, 빌드 파일 등으로 Log4j 사용 여부를 별도 확인하고, 사용 중이면 취약 버전이 포함되지 않도록 최신 보안 버전으로 유지한다.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1051,7 +1061,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1086,19 +1096,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 수집된 HTML 샘플에는 /vulnapp/css/style.css만 확인되고 jQuery 스크립트 로드 경로나 버전 문자열은 확인되지 않음. 시그니처 기반 보조 근거에서도 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상 여부를 확정할 수 없음. 시그니처 기반 추가 근거: 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 시그니처 기반 보조 근거에서 주요 페이지 HTML에서 jQuery 참조가 확인되지 않았고, collected_evidence의 /vulnapp/search.jsp 본문 샘플에도 jQuery 로드 경로나 버전 정보가 없다. 현재 수집 범위에서는 jQuery 사용 근거가 없어 n/a로 판단한다. 시그니처 기반 추가 근거: 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>전체 HTML 및 정적 리소스에서 jQuery 사용 여부와 버전을 식별하고, 사용 중이면 최신 지원 버전으로 업데이트하라. 미사용 라이브러리는 제거하라.</t>
+          <t>향후 jQuery를 도입하거나 별도 정적 리소스에서 사용이 확인될 경우 최신 안정 버전을 사용하고 알려진 취약 버전 여부를 점검한다.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1108,7 +1118,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1138,24 +1148,24 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>http://15.164.60.79/ 는 상태코드 200으로 HTTP 서비스가 제공됨. https://15.164.60.79 접속은 443 포트 연결 타임아웃으로 실패했고, https_available=false 및 redirect_to_https=false로 수집되어 HTTPS 제공 및 HTTP에서 HTTPS로의 강제 전환이 확인되지 않음. 시그니처 기반 추가 근거: HTTP 접속 가능 및 HTTPS 강제 리다이렉트 미확인. https_available=False, redirect_to_https=False</t>
+          <t>http://15.164.60.79/는 status_code 200으로 서비스되지만, https://15.164.60.79 접속은 443 포트 연결 타임아웃이 발생했다. 수집 데이터의 https_status에서 https_available=false, redirect_to_https=false로 확인된다. 시그니처 기반 추가 근거: HTTP 접속 가능 및 HTTPS 강제 리다이렉트 미확인. https_available=False, redirect_to_https=False</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>TLS 인증서를 적용하여 HTTPS 서비스를 제공하고 모든 HTTP 요청을 HTTPS로 리다이렉트하라. 인증, 세션, 개인정보 및 관리 기능은 HTTPS에서만 동작하도록 구성하라.</t>
+          <t>유효한 TLS 인증서를 적용하여 HTTPS 서비스를 활성화하고, HTTP 요청은 HTTPS로 리다이렉트한다. 적용 후 HSTS 설정을 검토한다.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1165,7 +1175,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1200,19 +1210,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>로그인 관련 응답의 Set-Cookie가 "JSESSIONID=...; Path=/vulnapp; HttpOnly"로 확인되어 HttpOnly는 설정되어 있으나 Secure 속성이 없음. XSS 테스트 중 발급된 JSESSIONID도 HttpOnly만 있고 Secure가 없음. 단순 GET 경로에서는 Set-Cookie가 없어 평가 대상 쿠키가 없었음. 시그니처 기반 추가 근거: Set-Cookie=JSESSIONID=93C56C9BE7DD0141A1C3A844302214F6; Path=/vulnapp; HttpOnly, missing=['secure', 'samesite']</t>
+          <t>SQL Injection 테스트 및 관리자 페이지 익명 요청에서 Set-Cookie: JSESSIONID=...; Path=/vulnapp; HttpOnly가 확인되었다. HttpOnly는 설정되어 있으나 Secure 속성이 없고, HTTPS가 사용 불가한 상태에서 HTTP로 세션 쿠키가 발급된다. 시그니처 기반 추가 근거: Set-Cookie=JSESSIONID=106B03824FD72B4B8716ABD2868EB7C6; Path=/vulnapp; HttpOnly, missing=['secure', 'samesite']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>HTTPS 적용 후 세션 쿠키에 Secure, HttpOnly, SameSite 속성을 명시하라. 인증 쿠키가 평문 HTTP로 전송되지 않도록 Secure를 반드시 적용하라.</t>
+          <t>HTTPS를 적용한 뒤 세션 쿠키에 Secure, HttpOnly, SameSite 속성을 명시적으로 설정한다. HTTP 환경에서 세션 쿠키가 발급되지 않도록 보안 설정을 강화한다.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1222,7 +1232,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1257,19 +1267,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>/vulnapp/login.jsp에 SQL Injection 인증 우회성 입력을 전송했을 때 세 차례 모두 상태코드 302와 Location: http://15.164.60.79/vulnapp/admin.jsp가 반환되고 JSESSIONID가 발급됨. SQL 오류 본문은 없으나 인증 우회성 리다이렉트 반응이 반복 확인됨. 시그니처 기반 보조 근거의 sqlmap 요약에서는 returncode 0으로 실행되었으나 dbms_banner, current_user, current_db, databases 정보는 식별되지 않았고, error_based는 false이며 auth_bypass는 true로 보고됨. 시그니처 기반 추가 근거: payload=' OR '1'='1' --, error_based=False, auth_bypass=True</t>
+          <t>SQL Injection 인증 우회 테스트에서 id 값에 "' OR '1'='1' -- ", "admin' -- ", "' OR 1=1 -- "를 입력하고 pw=test를 전송한 결과, 세 요청 모두 status_code 302로 응답하며 Location 헤더가 http://15.164.60.79/vulnapp/admin.jsp로 설정되었다. 이는 SQL 조건 조작으로 로그인 후 관리자 페이지로 이동된 정황이다. 시그니처 기반 보조 근거의 sqlmap_summary에 해당하는 정보로 sqlmap 실행 returncode는 0이었으나 dbms_banner, current_user, current_db, databases 정보는 null로 식별되지 않았다. 시그니처 기반 추가 근거: payload=' OR '1'='1' --, error_based=False, auth_bypass=True</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>로그인 쿼리를 Prepared Statement와 파라미터 바인딩으로 구현하고 사용자 입력을 SQL 문자열에 직접 결합하지 말라. 인증 성공 조건을 서버 측에서 엄격히 검증하고 관련 로그와 영향 범위를 점검하라.</t>
+          <t>로그인 쿼리에 Prepared Statement와 파라미터 바인딩을 적용하고 문자열 결합 방식의 SQL 생성을 제거한다. 인증 성공 조건을 명확히 검증하고, SQL 오류 및 인증 우회 테스트에 대한 보안 테스트를 추가한다.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1279,7 +1289,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1309,24 +1319,24 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>/vulnapp/search.jsp의 실제 파라미터 keyword에 입력한 값이 HTML 인코딩 없이 응답에 반사됨. keyword=&lt;script&gt;alert(1)&lt;/script&gt; 요청에서 value="&lt;script&gt;alert(1)&lt;/script&gt;" 및 &lt;strong&gt;'&lt;script&gt;alert(1)&lt;/script&gt;'&lt;/strong&gt; 형태로 출력되었고, keyword=\"&gt;&lt;script&gt;alert(1)&lt;/script&gt; 요청에서는 value=""&gt;&lt;script&gt;alert(1)&lt;/script&gt;" 형태로 속성 탈출 가능한 문자열이 반사됨. &lt;img src=x onerror=alert(1)&gt;도 인코딩 없이 반사됨. 시그니처 기반 추가 근거: keyword 파라미터에 입력한 script 태그가 응답에 HTML escaping 없이 반영됨.</t>
+          <t>/vulnapp/search.jsp의 keyword 파라미터에 &lt;script&gt;alert(1337)&lt;/script&gt;를 전달한 요청이 status_code 200으로 응답했고, 본문에 input value="&lt;script&gt;alert(1337)&lt;/script&gt;" 및 &lt;strong&gt;'&lt;script&gt;alert(1337)&lt;/script&gt;'&lt;/strong&gt; 형태로 HTML 이스케이프 없이 반사되었다. 다른 페이로드 "&gt;&lt;script&gt;alert(1)&lt;/script&gt;, &lt;img src=x onerror=alert(1)&gt;도 그대로 반사되었다. 시그니처 기반 추가 근거: keyword 파라미터에 입력한 script 태그가 응답에 HTML escaping 없이 반영됨.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>keyword 출력 시 HTML 본문, 속성 등 출력 컨텍스트에 맞는 인코딩을 적용하고 사용자 입력을 HTML에 직접 삽입하지 말라. 입력 검증과 함께 CSP를 보조 통제로 적용하라.</t>
+          <t>keyword 등 사용자 입력을 HTML 컨텍스트에 맞게 출력 인코딩하고, 속성 값에는 따옴표와 꺾쇠괄호 등을 안전하게 이스케이프한다. 입력 검증과 Content-Security-Policy를 병행 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1336,7 +1346,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1366,24 +1376,24 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>GPT 1차 판단은 저장 및 재조회 검증 데이터가 없어 보류였음. 시그니처 기반 보조 근거에서는 게시글 목록에서 저장형 XSS 페이로드 실행 흔적이 확인되지 않았다고 보고됨. collected_evidence에는 반사형 XSS는 확인되지만 저장형 입력 지점에 페이로드가 저장되어 다른 페이지나 세션에서 재출력된 증거는 없어, 현재 수집 범위에서는 Stored XSS 확인 안 됨으로 판단함. 시그니처 기반 추가 근거: 게시글 목록에서 저장형 XSS 페이로드 실행 흔적이 확인되지 않음. 상세 조회는 수동으로 추가 확인 필요.</t>
+          <t>수집 데이터에는 검색 파라미터가 즉시 응답에 반사되는 Reflected XSS 증거는 있으나, 게시글/프로필/업로드 등 저장 지점에 페이로드를 등록한 뒤 재조회하여 지속적으로 실행되는지 확인한 증거가 없다. 시그니처 기반 보조 근거도 저장된 게시글 상세 조회 검증이 필요하다고 보고하여 최종 판단을 보류한다. 시그니처 기반 추가 근거: 게시글 목록에서는 저장형 XSS 페이로드 실행 흔적이 확인되지 않았으나, 저장된 게시글 상세 조회 검증이 필요함. 수동진단에서 게시글 상세 조회 404가 확인되어 최종 판단 보류.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>게시글, 프로필, 업로드 메타데이터 등 모든 저장 데이터 출력 지점에 HTML escaping을 유지하고, 저장형 입력 지점이 추가될 경우 저장 후 재조회 기준으로 재점검하라.</t>
+          <t>입력 저장 기능이 있는 게시판, 프로필, 댓글, 업로드 메타데이터 등에 대해 저장 후 다른 세션에서 재조회하여 Stored XSS 여부를 검증한다. 저장 데이터 출력 시 컨텍스트별 인코딩을 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1393,7 +1403,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1423,24 +1433,24 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. /vulnapp/ping.jsp는 상태코드 404로 Not Found 응답이 확인되어 명령 실행 기능이 확인되지 않음. 명령 실행 파라미터, 지연 반응, 명령 출력 등 Command Injection 판단 근거가 없음. 시그니처 기반 추가 근거: /vulnapp/ping.jsp가 404로 확인되어 Command Injection 진단 대상 기능이 없음.</t>
+          <t>Command Injection 점검 대상으로 볼 수 있는 /vulnapp/ping.jsp는 optional_endpoint_status에서 status_code 404 Not Found로 응답했다. 수집 데이터에 명령 실행 기능이 있는 다른 엔드포인트나 파라미터는 확인되지 않아 현재 범위에서는 진단 대상 기능이 없는 것으로 판단한다. 시그니처 기반 추가 근거: /vulnapp/ping.jsp?host=127.0.0.1 요청이 404로 확인되어 Command Injection 진단을 수행할 수 없음.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>실제 명령 실행 기능이 존재하는 엔드포인트를 식별한 뒤 OS 명령 직접 호출을 제거하고, 불가피한 경우 허용 목록 기반 입력 검증과 안전한 API 사용을 적용하라.</t>
+          <t>명령 실행 기능이 존재하거나 향후 구현되는 경우 서버 측 명령 호출을 지양하고, 필요한 경우 허용 목록 기반 입력 검증과 안전한 API를 사용한다.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1450,7 +1460,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1485,19 +1495,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>rate_limit 수집 데이터에서 /vulnapp/login.jsp에 10회 시도한 결과 blocked=false로 기록됨. 각 시도는 상태코드 200을 반환했고 차단, 지연, 429 등 제한 응답 근거가 없음. 시그니처 기반 추가 근거: 잘못된 비밀번호 10회 연속 요청 상태코드: [200, 200, 200, 200, 200, 200, 200, 200, 200, 200]. 제한 응답 미확인.</t>
+          <t>rate_limit 수집 결과 /vulnapp/login.jsp에 대해 10회 로그인 시도 후 blocked=false로 기록되었고, 각 시도는 status_code 200으로 로그인 페이지가 계속 응답되었다. 차단, 지연, CAPTCHA 또는 429 응답 등의 제한 근거가 확인되지 않는다. 시그니처 기반 추가 근거: 잘못된 비밀번호 10회 연속 요청 상태코드: [200, 200, 200, 200, 200, 200, 200, 200, 200, 200]. 제한 응답 미확인.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>로그인 실패에 대해 IP, 계정, 세션 단위의 점진적 지연, 임시 차단, CAPTCHA 또는 429 응답 등 rate limiting 정책을 적용하라.</t>
+          <t>계정, IP, 세션, 디바이스 기준의 단계적 로그인 시도 제한을 적용하고 반복 실패 시 지연, CAPTCHA, 임시 차단, 모니터링 알림을 도입한다.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1507,7 +1517,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1542,19 +1552,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>account_lockout 수집 데이터에서 /vulnapp/login.jsp에 10회 시도 후 blocked=false로 기록됨. 모든 시도에서 상태코드 200 응답이 반환되었고 계정 잠금 또는 추가 인증 요구 근거가 없음. 시그니처 기반 추가 근거: 동일 계정 10회 실패 후에도 잠금/차단 응답 없음. statuses=[200, 200, 200, 200, 200, 200, 200, 200, 200, 200]</t>
+          <t>account_lockout 수집 결과 /vulnapp/login.jsp에 대해 10회 인증 시도 후 blocked=false로 기록되었으며, 모든 시도에서 status_code 200 응답이 계속 반환되었다. 계정 잠금 또는 임시 제한이 발생했다는 응답이 확인되지 않는다. 시그니처 기반 추가 근거: 동일 계정 10회 실패 후에도 잠금/차단 응답 없음. statuses=[200, 200, 200, 200, 200, 200, 200, 200, 200, 200]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>반복 인증 실패에 대해 계정 단위 임시 잠금, 위험 기반 추가 인증, 관리자 알림 및 감사 로그를 적용하라. 잠금 정책은 계정 열거와 서비스 거부 위험을 고려해 설계하라.</t>
+          <t>동일 계정에 대한 연속 로그인 실패 횟수를 제한하고, 임계치 초과 시 일정 시간 잠금 또는 추가 인증을 요구한다. 잠금 정책은 사용자 열거를 유발하지 않도록 일관된 메시지로 구현한다.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1564,7 +1574,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1594,24 +1604,24 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. /vulnapp/register.jsp는 상태코드 404로 확인되어 회원가입 기능이 확인되지 않았고, 비밀번호 변경 기능이나 약한 비밀번호 제출 결과도 수집되지 않음. 따라서 약한 비밀번호 허용 여부를 판단할 수 없음. 시그니처 기반 추가 근거: /vulnapp/register.jsp가 404로 확인되어 약한 비밀번호 정책 진단 대상 기능이 없음.</t>
+          <t>수집 데이터에는 회원가입 또는 비밀번호 변경 요청/응답, 약한 비밀번호 입력 테스트 결과가 없다. /vulnapp/register.jsp는 status_code 404로 확인되어 비밀번호 정책 판단에 필요한 기능 응답이 없다. 시그니처 기반 보조 근거도 해당 기능 404로 진단 불가를 보고하므로 최종 판단을 보류한다. 시그니처 기반 추가 근거: /vulnapp/register.jsp 요청이 404로 확인되어 약한 비밀번호 허용 여부를 진단할 수 없음.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>회원가입 및 비밀번호 변경 기능에서 최소 길이, 복잡도, 유출 비밀번호 차단, 사용자 정보 포함 금지 등 정책 적용 여부를 점검하라.</t>
+          <t>회원가입, 비밀번호 변경, 초기화 기능에서 최소 길이, 복잡도, 사전/유출 비밀번호 차단 등 정책이 적용되는지 테스트한다. 기능 구현 후 서버 측 검증을 반드시 적용한다.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1621,7 +1631,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1646,7 +1656,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>/vulnapp/login.jsp</t>
+          <t>/vulnapp/</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1656,19 +1666,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 인증 관련 응답은 JSESSIONID 세션 쿠키 발급이며 JWT, Authorization Bearer 헤더, access_token 등 JWT 사용 근거가 확인되지 않음. JWT 미사용으로 검증 우회 여부를 판단할 수 없음. 시그니처 기반 추가 근거: 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않음.</t>
+          <t>수집된 인증 관련 응답은 JSESSIONID 세션 쿠키 기반이며, Authorization: Bearer 토큰이나 JWT 형식의 토큰이 응답 헤더/쿠키/본문에서 확인되지 않는다. 현재 수집 범위에서는 JWT 사용 근거가 없어 진단 대상이 아니다. 시그니처 기반 추가 근거: 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않음.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>JWT를 사용하는 API가 존재하는지 확인하고, 도입 시 서명 검증, alg=none 차단, 만료 검증, 키 관리 및 클레임 검증을 적용하라.</t>
+          <t>JWT를 사용하는 API가 별도로 존재한다면 alg=none, 서명 검증 우회, 만료 검증 누락 등을 추가 점검한다. 현재 확인된 세션 기반 인증에는 해당 항목이 적용되지 않는다.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1678,7 +1688,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1708,24 +1718,24 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. /vulnapp/upload.jsp는 상태코드 200으로 접근 가능하고 /vulnapp/upload_process.jsp는 상태코드 500 응답이 확인되었으나, JSP 또는 스크립트 파일 업로드 시도, 저장 경로, 실행 가능 여부에 대한 응답 데이터가 없음. 웹쉘 업로드 가능 여부를 확정할 근거가 부족함. 시그니처 기반 추가 근거: JSP 업로드 실행 여부가 확인되지 않음. 업로드 처리 오류 또는 저장 경로 확인 필요.</t>
+          <t>/vulnapp/upload.jsp는 status_code 200으로 접근 가능하고 /vulnapp/upload_process.jsp는 status_code 500 응답이 확인되지만, 실제 파일 업로드 요청, JSP 파일 업로드 성공 여부, 웹 경로에서 JSP 실행 가능 여부에 대한 수집 데이터가 없다. 시그니처 기반 보조 근거도 업로드 실행 여부가 확인되지 않았다고 보고하므로 최종 판단을 보류한다. 시그니처 기반 추가 근거: shell.jsp 업로드 시도 후 업로드 실행 여부가 확인되지 않음. upload_process.jsp 500, 저장 경로 404 등 업로드 처리 오류 또는 저장 경로 확인이 필요함.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>업로드 기능에 허용 확장자, MIME/매직바이트 검증, 파일명 무작위화, 웹루트 외부 저장, 실행 권한 제거를 적용하고 업로드 성공/거부 결과가 명확히 반환되도록 구현하라.</t>
+          <t>업로드 기능에 확장자/콘텐츠 타입/매직바이트 검증, 저장 경로 실행 권한 제거, 파일명 난수화, 악성 파일 검사, 업로드 후 직접 실행 차단을 적용하고 실제 업로드 및 실행 차단 여부를 재검증한다.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1735,7 +1745,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1760,29 +1770,29 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>/vulnapp/profile.jsp</t>
+          <t>/vulnapp/upload_process.jsp</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>GPT 1차 판단은 /vulnapp/upload_process.jsp의 일부 500 응답 샘플에서 상세 스택 트레이스가 확인되지 않아 보류였음. 시그니처 기반 보조 근거에서는 /vulnapp/profile.jsp?user_idx=abc 응답에 내부 DB/예외 메시지가 노출된 것으로 보고됨. collected_evidence와 점검 URL이 달라 직접 본문 검증에는 한계가 있으나, 예외 처리 정보 노출 가능성이 있어 보수적으로 낮은 심각도의 취약으로 판단함. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/profile.jsp?user_idx=abc 응답에 내부 DB/예외 메시지 노출</t>
+          <t>/vulnapp/upload_process.jsp 요청이 status_code 500으로 응답했고 Tomcat 기본 오류 페이지 일부가 수집되었으나, 제공된 body_sample에는 Java 예외 클래스명, stack trace 프레임, 소스 파일/라인 번호 등 상세 스택 트레이스 노출 근거가 포함되어 있지 않다. 시그니처 기반 보조 근거도 내부 DB/예외 메시지 가능성은 언급하지만 Java/Tomcat stack trace 자체는 확인되지 않았다고 보고하여 최종 판단을 보류한다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/profile.jsp?user_idx=abc 응답에 내부 DB/예외 메시지가 노출되지만 Java/Tomcat stack trace 자체는 확인되지 않음. 원래 양호 항목으로 설계되어 사이트 수정 후 재진단 필요.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>사용자 응답에는 일반화된 오류 메시지만 표시하고 상세 예외, DB 오류, 스택 트레이스, 소스 파일명과 라인 번호는 서버 로그에만 기록하라. 입력값 타입 검증과 전역 예외 처리 페이지를 적용하라.</t>
+          <t>500 오류 발생 시 사용자에게는 일반화된 오류 페이지를 제공하고, 상세 예외와 스택 트레이스는 서버 로그에만 기록한다. 전체 오류 응답을 확인하여 스택 트레이스 노출 여부를 추가 점검한다.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SCAN-20260517-171315</t>
+          <t>SCAN-20260517-185902</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1792,7 +1802,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-05-17T17:13:15+09:00</t>
+          <t>2026-05-17T18:59:02+09:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1822,17 +1832,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. /vulnapp/fetch.jsp는 상태코드 404로 Not Found 응답이 확인되어 SSRF 대상인 서버 측 URL 요청 기능이 확인되지 않음. 외부 URL 입력, 내부 주소 요청 결과, 타임아웃 또는 블라인드 SSRF 반응 데이터가 없어 SSRF 여부를 판단할 수 없음. 시그니처 기반 추가 근거: /vulnapp/fetch.jsp가 404로 확인되어 SSRF 진단 대상 기능이 없음.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에서 SSRF 점검 대상으로 볼 수 있는 /vulnapp/fetch.jsp는 status_code 404 Not Found로 응답했고, 외부 URL을 서버가 가져오는 기능이나 관련 파라미터 응답은 확인되지 않는다. 시그니처 기반 보조 근거도 /vulnapp/fetch.jsp와 내부 테스트 자원이 404로 확인되어 SSRF 진단을 수행할 수 없다고 보고하므로 최종 판단을 보류한다. 시그니처 기반 추가 근거: /vulnapp/fetch.jsp가 404로 확인되어 SSRF 진단을 수행할 수 없음. /vulnapp/internal/secret.jsp도 404라 내부 테스트 자원 확인이 필요함.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>URL fetch, webhook, 이미지 프록시 등 서버 측 요청 기능이 존재하는 경우 내부 IP와 메타데이터 주소 차단, DNS rebinding 방어, 허용 목록 기반 목적지 검증, 응답 크기 및 타임아웃 제한을 적용하라.</t>
+          <t>URL fetch, webhook, 이미지 프록시 등 서버 측 요청 기능이 존재하거나 구현 예정이면 내부 IP 및 메타데이터 주소 접근 차단, 허용 목록, 리다이렉트 제한, DNS rebinding 방어를 적용하고 기능 정상화 후 재진단한다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix webshell detection and update scan results
</commit_message>
<xml_diff>
--- a/auto-scanner/outputs/자동진단.xlsx
+++ b/auto-scanner/outputs/자동진단.xlsx
@@ -445,7 +445,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -586,7 +586,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="51" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="80" customWidth="1" min="10" max="10"/>
     <col width="80" customWidth="1" min="11" max="11"/>
@@ -652,7 +652,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -697,19 +697,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>익명 요청은 /vulnapp/admin.jsp에서 302로 /vulnapp/login.jsp로 리다이렉트되었으나, 일반 사용자 계정(user1) 로그인 후 동일한 /vulnapp/admin.jsp 요청이 status_code 200으로 응답하였다. 응답 본문에 "⚙️ 시스템 관리자 대시보드", "Admin Only", "현재 서버에 가입된 모든 회원" 문구가 포함되어 일반 사용자가 관리자 전용 페이지에 접근 가능한 것으로 확인된다. 시그니처 기반 추가 근거: /vulnapp/admin.jsp 비로그인 요청은 로그인 페이지로 리다이렉트됨. 일반 사용자(user1) 로그인 세션으로 /vulnapp/admin.jsp 접근 시 200 응답과 관리자 페이지 키워드가 확인되어 관리자 권한 검증 미흡이 확인됨.</t>
+          <t>익명 요청은 /vulnapp/admin.jsp에서 302로 /vulnapp/login.jsp로 리다이렉트되어 비로그인 접근은 차단되었으나, 일반 사용자 user1 로그인 후 동일한 관리자 페이지 요청이 200으로 응답되었고 본문에 '시스템 관리자 대시보드', 'Admin Only', '현재 서버에 가입된 모든 회원' 문구가 포함되었다. 일반 사용자 세션으로 관리자 전용 페이지 접근이 가능하므로 권한 검증 미흡으로 판단한다. 시그니처 기반 추가 근거: /vulnapp/admin.jsp 비로그인 요청은 로그인 페이지로 리다이렉트됨. 일반 사용자(user1) 로그인 세션으로 /vulnapp/admin.jsp 접근 시 200 응답과 관리자 페이지 키워드가 확인되어 관리자 권한 검증 미흡이 확인됨.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>관리자 기능은 서버 측에서 사용자 역할/권한을 검증하여 관리자 권한이 없는 세션은 403 처리하거나 접근을 차단해야 한다. 모든 관리자 페이지와 API에 동일한 권한 검사를 적용한다.</t>
+          <t>관리자 기능은 인증 여부뿐 아니라 관리자 역할/권한을 서버 측에서 검증해야 한다. /vulnapp/admin.jsp 접근 시 세션의 role 또는 authority를 확인하고 일반 사용자는 403 또는 접근 권한 없음 페이지로 차단하라.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -754,19 +754,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 시그니처 기반 보조 근거에 따르면 profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출되는 것으로 보고되었다. collected_evidence에는 /vulnapp/profile.jsp?user_idx=1의 200 응답만 있고 사용자 간 비교 본문은 부족하므로, 시그니처 결과를 보조 근거로 최종 취약 판단한다. 시그니처 기반 추가 근거: profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출됨.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/profile.jsp?user_idx=1이 200으로 도달 가능하다는 정보만 있어 단독으로는 IDOR 여부를 확정하기 부족했으나, 시그니처 기반 보조 근거에서 profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출된 것으로 보고되었다. 시그니처 기반 추가 근거: profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출됨.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>사용자 정보 조회 시 세션 사용자와 조회 대상 객체의 소유자 또는 권한을 서버 측에서 검증하고, 권한 없는 user_idx 접근은 403 또는 일반화된 오류로 차단해야 한다.</t>
+          <t>사용자 정보 조회 시 요청 파라미터의 user_idx만 신뢰하지 말고 세션 사용자와 조회 대상의 소유자 또는 접근 권한을 서버 측에서 검증하라. 권한 없는 객체 접근은 403으로 차단하고 식별자는 예측 가능성을 낮추는 방식을 검토하라.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/vulnapp/</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>기본 페이지 http://15.164.60.79/ 응답 헤더에서 Content-Security-Policy, X-Frame-Options 또는 frame-ancestors, X-Content-Type-Options, Referrer-Policy, Strict-Transport-Security 등의 주요 보안 헤더가 확인되지 않는다. 시그니처 기반 추가 근거: /vulnapp/ 응답에서 주요 보안 헤더 누락: ['Content-Security-Policy', 'X-Frame-Options', 'X-Content-Type-Options', 'Referrer-Policy']</t>
+          <t>/vulnapp/의 200 응답 헤더에는 Server, Date, Content-Type, Transfer-Encoding, Connection, Set-Cookie, Content-Encoding만 확인되며 Content-Security-Policy, X-Frame-Options, X-Content-Type-Options, Referrer-Policy, Strict-Transport-Security 등의 주요 보안 헤더가 확인되지 않는다. 시그니처 기반 추가 근거: /vulnapp/ 응답에서 주요 보안 헤더 누락: ['Content-Security-Policy', 'X-Frame-Options', 'X-Content-Type-Options', 'Referrer-Policy']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Content-Security-Policy, X-Frame-Options 또는 CSP frame-ancestors, X-Content-Type-Options: nosniff, Referrer-Policy, Permissions-Policy 등을 설정한다. HTTPS 적용 후 HSTS도 설정한다.</t>
+          <t>애플리케이션 또는 nginx에서 Content-Security-Policy, X-Frame-Options 또는 frame-ancestors, X-Content-Type-Options: nosniff, Referrer-Policy 등을 설정하라. HTTPS 적용 후 HSTS도 설정하라.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/vulnapp/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -868,19 +868,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>http://15.164.60.79/ 응답 헤더에 "Server: nginx/1.28.3 (Ubuntu)"가 노출된다. 또한 기본 페이지 본문 title 및 h1, 404 오류 페이지 하단에 "Apache Tomcat/9.0.118"가 노출된다. 시그니처 기반 추가 근거: http://15.164.60.79/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79/ body contains Apache Tomcat/; http://15.164.60.79/vulnapp/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79:8080/ body contains Apache Tomcat/</t>
+          <t>/vulnapp/ 및 404 응답의 Server 헤더가 'nginx/1.28.3 (Ubuntu)'로 제품명, 버전, OS 정보를 노출한다. 또한 / 및 :8080/의 Tomcat 기본 페이지 본문 title/h1에 'Apache Tomcat/9.0.118' 버전이 표시된다. 시그니처 기반 추가 근거: http://15.164.60.79/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79/ body contains Apache Tomcat/; http://15.164.60.79/vulnapp/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79:8080/ body contains Apache Tomcat/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>nginx의 server_tokens를 비활성화하고, Tomcat 기본/오류 페이지에서 제품명 및 상세 버전이 노출되지 않도록 커스텀 오류 페이지와 배너 제거 설정을 적용한다.</t>
+          <t>nginx server_tokens off 설정 등으로 상세 버전 노출을 제거하고, Tomcat 기본 페이지와 오류 페이지에서 제품명 및 상세 버전 정보가 노출되지 않도록 설정하라.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -925,19 +925,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>http://15.164.60.79:8080/ 및 http://15.164.60.79/ 요청이 status_code 200으로 응답했고, 본문에 "Apache Tomcat/9.0.118", "If you're seeing this, you've successfully installed Tomcat. Congratulations!", /docs/, /examples/ 링크 등 Tomcat 기본 페이지 내용이 확인된다. 시그니처 기반 추가 근거: http://15.164.60.79:8080/에서 Tomcat 기본 페이지와 Manager/Host Manager 링크 노출</t>
+          <t>http://15.164.60.79/ 및 http://15.164.60.79:8080/ 요청이 200으로 응답되며 본문에 '&lt;title&gt;Apache Tomcat/9.0.118&lt;/title&gt;', '&lt;h1&gt;Apache Tomcat/9.0.118&lt;/h1&gt;', 'If you're seeing this, you've successfully installed Tomcat. Congratulations!'가 포함된 Tomcat 기본 페이지가 노출된다. 시그니처 기반 추가 근거: http://15.164.60.79:8080/에서 Tomcat 기본 페이지와 Manager/Host Manager 링크 노출</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>운영 환경에서는 Tomcat ROOT 기본 애플리케이션, docs, examples 등 불필요한 기본 리소스를 제거하고 실제 서비스 페이지 또는 차단 페이지로 대체한다. 8080 포트의 외부 노출 필요성도 재검토한다.</t>
+          <t>운영 환경에서는 Tomcat ROOT 기본 애플리케이션, docs, examples 등 기본 리소스를 제거하거나 접근을 차단하고 필요한 애플리케이션만 배포하라. 8080 포트의 외부 접근 제한도 검토하라.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -982,19 +982,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>http://15.164.60.79/vulnapp/debug.jsp와 /vulnapp/debug.jsp?debug=true가 모두 status_code 200, Content-Type application/json으로 응답했다. 본문에 "debug": true와 함께 "db_user": "vulnuser", "db_password": "vulnpass1234", "api_key": "TEST-API-KEY-123456", "internal_ip": "10.0.0.5"가 노출된다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/debug.jsp에서 debug/API 키/DB 계정/내부 IP 등 내부 정보 노출</t>
+          <t>/vulnapp/debug.jsp 및 /vulnapp/debug.jsp?debug=true가 200, Content-Type application/json으로 응답하며 본문에 'debug: true', db_user 'vulnuser', db_password 'vulnpass1234', api_key 'TEST-API-KEY-123456', internal_ip '10.0.0.5'가 노출된다. 이번 프로젝트 기준에 따라 medium으로 판단한다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/debug.jsp에서 debug/API 키/DB 계정/내부 IP 등 내부 정보 노출</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>운영 환경에서 debug 기능과 debug 엔드포인트를 비활성화하거나 인증/인가된 관리자에게만 제한한다. 노출된 DB 계정 비밀번호와 API 키는 즉시 폐기 및 재발급하고, 민감정보가 응답에 포함되지 않도록 제거한다.</t>
+          <t>운영 환경에서 debug 엔드포인트와 debug=true 기능을 비활성화하고 인증/인가를 적용하라. 노출된 DB 계정 비밀번호와 API 키는 즉시 폐기 및 재발급하라.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>/vulnapp/</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1039,19 +1039,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 시그니처 기반 보조 근거에서 외부 HTTP 응답상 Log4j 사용 흔적이 확인되지 않았고, collected_evidence에도 Log4j 라이브러리나 취약 버전을 판단할 근거가 없다. 현재 외부 진단 범위에서는 진단 대상 기능 또는 사용 흔적이 확인되지 않아 n/a로 판단한다. 시그니처 기반 추가 근거: 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않음. 서버 내부 라이브러리 확인은 수동진단으로 보완 필요.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 Log4j 라이브러리 사용 여부, 버전, 의존성 목록이 없었으며, 시그니처 기반 보조 근거에서도 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않았다. 현재 외부 진단 범위에서는 해당 기술 사용 증거가 없어 진단 대상 아님으로 판단한다. 시그니처 기반 추가 근거: 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않음. 서버 내부 라이브러리 확인은 수동진단으로 보완 필요.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>서버 내부 SBOM, WEB-INF/lib, 빌드 파일 등으로 Log4j 사용 여부를 별도 확인하고, 사용 중이면 취약 버전이 포함되지 않도록 최신 보안 버전으로 유지한다.</t>
+          <t>서버 내부 의존성 목록 또는 배포 패키지에서 Log4j 사용 여부와 버전을 주기적으로 확인하라. 향후 Log4j를 도입하거나 사용 중인 사실이 확인되면 취약 버전 여부를 점검하고 안전한 최신 버전으로 업그레이드하라.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>/vulnapp/search.jsp</t>
+          <t>/vulnapp/</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1096,19 +1096,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 시그니처 기반 보조 근거에서 주요 페이지 HTML에서 jQuery 참조가 확인되지 않았고, collected_evidence의 /vulnapp/search.jsp 본문 샘플에도 jQuery 로드 경로나 버전 정보가 없다. 현재 수집 범위에서는 jQuery 사용 근거가 없어 n/a로 판단한다. 시그니처 기반 추가 근거: 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence의 HTML 샘플에는 /vulnapp/css/style.css 링크만 확인되고 jQuery 스크립트 경로나 버전 정보가 없었다. 시그니처 기반 보조 근거에서도 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아닌 것으로 보고되었다. 시그니처 기반 추가 근거: 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>향후 jQuery를 도입하거나 별도 정적 리소스에서 사용이 확인될 경우 최신 안정 버전을 사용하고 알려진 취약 버전 여부를 점검한다.</t>
+          <t>향후 jQuery를 도입하는 경우 보안 지원되는 최신 버전을 사용하고, SCA 도구나 정적 리소스 점검으로 취약 버전 사용 여부를 주기적으로 확인하라.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1153,19 +1153,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>http://15.164.60.79/는 status_code 200으로 서비스되지만, https://15.164.60.79 접속은 443 포트 연결 타임아웃이 발생했다. 수집 데이터의 https_status에서 https_available=false, redirect_to_https=false로 확인된다. 시그니처 기반 추가 근거: HTTP 접속 가능 및 HTTPS 강제 리다이렉트 미확인. https_available=False, redirect_to_https=False</t>
+          <t>http://15.164.60.79/는 200으로 응답하지만, https://15.164.60.79는 443 포트 연결 타임아웃으로 https_available=false이며 redirect_to_https=false로 기록되어 있다. HTTPS가 제공되지 않고 HTTP에서 HTTPS로 강제 전환되지 않아 이번 프로젝트 기준에 따라 medium으로 판단한다. 시그니처 기반 추가 근거: HTTP 접속 가능 및 HTTPS 강제 리다이렉트 미확인. https_available=False, redirect_to_https=False</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>유효한 TLS 인증서를 적용하여 HTTPS 서비스를 활성화하고, HTTP 요청은 HTTPS로 리다이렉트한다. 적용 후 HSTS 설정을 검토한다.</t>
+          <t>유효한 TLS 인증서를 적용하여 HTTPS 서비스를 활성화하고 모든 HTTP 요청을 HTTPS로 리다이렉트하라. 로그인, 세션 쿠키, 개인정보 등 민감 정보 전송 구간은 반드시 TLS로 보호하라.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>/vulnapp/login.jsp</t>
+          <t>/vulnapp/</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1210,19 +1210,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>SQL Injection 테스트 및 관리자 페이지 익명 요청에서 Set-Cookie: JSESSIONID=...; Path=/vulnapp; HttpOnly가 확인되었다. HttpOnly는 설정되어 있으나 Secure 속성이 없고, HTTPS가 사용 불가한 상태에서 HTTP로 세션 쿠키가 발급된다. 시그니처 기반 추가 근거: Set-Cookie=JSESSIONID=106B03824FD72B4B8716ABD2868EB7C6; Path=/vulnapp; HttpOnly, missing=['secure', 'samesite']</t>
+          <t>basic_page 응답의 Set-Cookie는 'JSESSIONID=...; Path=/vulnapp; HttpOnly'로 HttpOnly는 있으나 Secure 속성이 없다. SQL Injection 테스트 및 관리자 페이지 익명 요청의 JSESSIONID Set-Cookie도 Path=/vulnapp; HttpOnly만 포함하고 Secure가 없다. HTTPS가 미적용된 상태라 Secure 쿠키도 적용되지 않은 것으로 확인된다. 시그니처 기반 추가 근거: Set-Cookie=JSESSIONID=CB689639FD615B11C2C3EE1F1A8AAB44; Path=/vulnapp; HttpOnly, missing=['secure', 'samesite']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>HTTPS를 적용한 뒤 세션 쿠키에 Secure, HttpOnly, SameSite 속성을 명시적으로 설정한다. HTTP 환경에서 세션 쿠키가 발급되지 않도록 보안 설정을 강화한다.</t>
+          <t>HTTPS 적용 후 세션 쿠키에 Secure, HttpOnly, SameSite=Lax 또는 Strict 속성을 설정하라. 인증 쿠키가 평문 HTTP로 전송되지 않도록 HTTPS 강제 전환과 함께 적용하라.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1267,19 +1267,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>SQL Injection 인증 우회 테스트에서 id 값에 "' OR '1'='1' -- ", "admin' -- ", "' OR 1=1 -- "를 입력하고 pw=test를 전송한 결과, 세 요청 모두 status_code 302로 응답하며 Location 헤더가 http://15.164.60.79/vulnapp/admin.jsp로 설정되었다. 이는 SQL 조건 조작으로 로그인 후 관리자 페이지로 이동된 정황이다. 시그니처 기반 보조 근거의 sqlmap_summary에 해당하는 정보로 sqlmap 실행 returncode는 0이었으나 dbms_banner, current_user, current_db, databases 정보는 null로 식별되지 않았다. 시그니처 기반 추가 근거: payload=' OR '1'='1' --, error_based=False, auth_bypass=True</t>
+          <t>SQL Injection authentication bypass test에서 /vulnapp/login.jsp의 id 값에 조건 조작 입력을 전송한 3개 요청이 모두 302로 응답했고 Location 헤더가 http://15.164.60.79/vulnapp/admin.jsp로 설정되었다. 정상 인증 정보가 아닌 입력으로 관리자 페이지로 리다이렉트되는 반응이 확인된다. 시그니처 기반 보조 근거의 sqlmap 보조 점검에서도 인증 우회가 확인되었고, DBMS 배너는 MySQL 계열 MariaDB 11.8.6-MariaDB-5 from Ubuntu로 식별되었으며, 현재 DB 사용자는 vulnuser@localhost, 현재 데이터베이스는 vuln_db로 확인되었다. 열거된 데이터베이스는 information_schema와 vuln_db이고 현재 DB 계정은 DBA 권한은 아닌 것으로 보고되었다. 시그니처 기반 추가 근거: payload=' OR '1'='1' --, redirect_location=http://15.164.60.79/vulnapp/admin.jsp, error_based=False, auth_bypass=True, sqlmap 보조 점검 결과: DBMS 배너는 MySQL &gt;= 5.1 (MariaDB fork) / banner=11.8.6-MariaDB-5 from Ubuntu로 식별됨. DB 현재 사용자는 vulnuser@localhost로 확인됨. current database() 값은 vuln_db로 확인됨. 현재 DB 계정은 DBA 권한으로 식별되지 않음. 열거된 데이터베이스는 information_schema, vuln_db 임.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>로그인 쿼리에 Prepared Statement와 파라미터 바인딩을 적용하고 문자열 결합 방식의 SQL 생성을 제거한다. 인증 성공 조건을 명확히 검증하고, SQL 오류 및 인증 우회 테스트에 대한 보안 테스트를 추가한다.</t>
+          <t>로그인 쿼리에 Prepared Statement와 파라미터 바인딩을 사용하고 문자열 연결 방식의 SQL 생성을 제거하라. 인증 로직을 재검토하고 입력값 검증, DB 오류 메시지 비노출, 최소 권한 DB 계정 적용을 병행하라.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1324,19 +1324,19 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>/vulnapp/search.jsp의 keyword 파라미터에 &lt;script&gt;alert(1337)&lt;/script&gt;를 전달한 요청이 status_code 200으로 응답했고, 본문에 input value="&lt;script&gt;alert(1337)&lt;/script&gt;" 및 &lt;strong&gt;'&lt;script&gt;alert(1337)&lt;/script&gt;'&lt;/strong&gt; 형태로 HTML 이스케이프 없이 반사되었다. 다른 페이로드 "&gt;&lt;script&gt;alert(1)&lt;/script&gt;, &lt;img src=x onerror=alert(1)&gt;도 그대로 반사되었다. 시그니처 기반 추가 근거: keyword 파라미터에 입력한 script 태그가 응답에 HTML escaping 없이 반영됨.</t>
+          <t>/vulnapp/search.jsp의 실제 파라미터 keyword에 '&lt;script&gt;alert(1337)&lt;/script&gt;'를 전달한 응답에서 입력값이 input value 및 strong 태그 영역에 HTML 이스케이프 없이 반사되었다. 또한 '"&gt;&lt;script&gt;alert(1)&lt;/script&gt;' 입력 시 input value 속성 컨텍스트를 탈출한 스크립트 태그가 응답 본문에 포함되었다. 이번 프로젝트 기준에 따라 Reflected XSS는 medium으로 판단한다. 시그니처 기반 추가 근거: keyword 파라미터에 입력한 script 태그가 응답에 HTML escaping 없이 반영됨.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>keyword 등 사용자 입력을 HTML 컨텍스트에 맞게 출력 인코딩하고, 속성 값에는 따옴표와 꺾쇠괄호 등을 안전하게 이스케이프한다. 입력 검증과 Content-Security-Policy를 병행 적용한다.</t>
+          <t>검색어 등 사용자 입력을 출력 컨텍스트에 맞게 HTML 본문, HTML 속성, JavaScript 컨텍스트별로 인코딩하라. CSP를 적용하여 스크립트 실행 위험을 완화하고 입력 검증만이 아니라 출력 인코딩을 필수로 적용하라.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1371,29 +1371,29 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>/vulnapp/search.jsp</t>
+          <t>/vulnapp/board.jsp</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>수집 데이터에는 검색 파라미터가 즉시 응답에 반사되는 Reflected XSS 증거는 있으나, 게시글/프로필/업로드 등 저장 지점에 페이로드를 등록한 뒤 재조회하여 지속적으로 실행되는지 확인한 증거가 없다. 시그니처 기반 보조 근거도 저장된 게시글 상세 조회 검증이 필요하다고 보고하여 최종 판단을 보류한다. 시그니처 기반 추가 근거: 게시글 목록에서는 저장형 XSS 페이로드 실행 흔적이 확인되지 않았으나, 저장된 게시글 상세 조회 검증이 필요함. 수동진단에서 게시글 상세 조회 404가 확인되어 최종 판단 보류.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/board.jsp가 200으로 존재한다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 /vulnapp/board.jsp에 저장한 테스트 게시글을 재조회했을 때 script 페이로드가 HTML escape된 형태로만 확인되어 Stored XSS가 차단된 것으로 보고되었다. 시그니처 기반 추가 근거: /vulnapp/board.jsp에 저장한 테스트 게시글이 재조회되었고 script 페이로드가 HTML escape된 형태로만 확인되어 Stored XSS가 차단됨.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>입력 저장 기능이 있는 게시판, 프로필, 댓글, 업로드 메타데이터 등에 대해 저장 후 다른 세션에서 재조회하여 Stored XSS 여부를 검증한다. 저장 데이터 출력 시 컨텍스트별 인코딩을 적용한다.</t>
+          <t>현재 게시글 출력 인코딩 정책을 유지하고, 게시글 목록/상세/댓글/프로필 등 저장 데이터가 출력되는 모든 지점에 동일한 컨텍스트 기반 이스케이프를 적용하라.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1428,29 +1428,29 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>/vulnapp/ping.jsp</t>
+          <t>/vulnapp/command.jsp</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Command Injection 점검 대상으로 볼 수 있는 /vulnapp/ping.jsp는 optional_endpoint_status에서 status_code 404 Not Found로 응답했다. 수집 데이터에 명령 실행 기능이 있는 다른 엔드포인트나 파라미터는 확인되지 않아 현재 범위에서는 진단 대상 기능이 없는 것으로 판단한다. 시그니처 기반 추가 근거: /vulnapp/ping.jsp?host=127.0.0.1 요청이 404로 확인되어 Command Injection 진단을 수행할 수 없음.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/command.jsp가 200으로 도달 가능하다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 명령어 삽입 테스트 입력에 대해 실행 결과가 노출되지 않았고 관련 페이로드가 차단된 것으로 보고되어 현재 수집 범위에서는 방어된 항목으로 판단한다. 시그니처 기반 추가 근거: /vulnapp/command.jsp 명령어 삽입 페이로드에서 실행 결과 미노출. blocked=['time_snapshot;whoami', 'host_summary&amp;&amp;id', 'uptime_check|whoami']</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>명령 실행 기능이 존재하거나 향후 구현되는 경우 서버 측 명령 호출을 지양하고, 필요한 경우 허용 목록 기반 입력 검증과 안전한 API를 사용한다.</t>
+          <t>작업 코드나 상태 조회 입력값은 허용 목록 기반으로 검증하고 OS 명령 문자열에 사용자 입력을 직접 결합하지 말라. 가능한 경우 OS 명령 호출 대신 안전한 서버 API를 사용하라.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1495,19 +1495,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>rate_limit 수집 결과 /vulnapp/login.jsp에 대해 10회 로그인 시도 후 blocked=false로 기록되었고, 각 시도는 status_code 200으로 로그인 페이지가 계속 응답되었다. 차단, 지연, CAPTCHA 또는 429 응답 등의 제한 근거가 확인되지 않는다. 시그니처 기반 추가 근거: 잘못된 비밀번호 10회 연속 요청 상태코드: [200, 200, 200, 200, 200, 200, 200, 200, 200, 200]. 제한 응답 미확인.</t>
+          <t>rate_limit 수집 결과에서 /vulnapp/login.jsp에 대해 10회 연속 요청을 수행했으나 blocked=false이며 각 시도는 200으로 로그인 페이지 응답을 계속 반환했다. 차단, 지연, CAPTCHA, 429 응답 등의 제한 동작이 확인되지 않았다. 시그니처 기반 추가 근거: 잘못된 비밀번호 10회 연속 요청 상태코드: [200, 200, 200, 200, 200, 200, 200, 200, 200, 200]. 제한 응답 미확인.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>계정, IP, 세션, 디바이스 기준의 단계적 로그인 시도 제한을 적용하고 반복 실패 시 지연, CAPTCHA, 임시 차단, 모니터링 알림을 도입한다.</t>
+          <t>로그인 실패 횟수에 따른 IP/계정 기반 속도 제한, 지수 백오프, CAPTCHA 또는 일시 차단 정책을 적용하고 모니터링 및 알림을 구성하라.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1552,19 +1552,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>account_lockout 수집 결과 /vulnapp/login.jsp에 대해 10회 인증 시도 후 blocked=false로 기록되었으며, 모든 시도에서 status_code 200 응답이 계속 반환되었다. 계정 잠금 또는 임시 제한이 발생했다는 응답이 확인되지 않는다. 시그니처 기반 추가 근거: 동일 계정 10회 실패 후에도 잠금/차단 응답 없음. statuses=[200, 200, 200, 200, 200, 200, 200, 200, 200, 200]</t>
+          <t>account_lockout 수집 결과에서 /vulnapp/login.jsp에 대해 10회 시도 후에도 blocked=false이고 모든 시도 응답이 200으로 계속 반환되었다. 반복 실패 후 계정 잠금 또는 일시 차단 동작이 확인되지 않았다. 시그니처 기반 추가 근거: 동일 계정 10회 실패 후에도 잠금/차단 응답 없음. statuses=[200, 200, 200, 200, 200, 200, 200, 200, 200, 200]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>동일 계정에 대한 연속 로그인 실패 횟수를 제한하고, 임계치 초과 시 일정 시간 잠금 또는 추가 인증을 요구한다. 잠금 정책은 사용자 열거를 유발하지 않도록 일관된 메시지로 구현한다.</t>
+          <t>계정별 연속 로그인 실패 횟수 기준의 일시 잠금 또는 추가 인증 절차를 적용하라. 잠금 정책은 사용자 안내와 관리자 해제 또는 자동 해제 절차를 포함해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1604,24 +1604,24 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>수집 데이터에는 회원가입 또는 비밀번호 변경 요청/응답, 약한 비밀번호 입력 테스트 결과가 없다. /vulnapp/register.jsp는 status_code 404로 확인되어 비밀번호 정책 판단에 필요한 기능 응답이 없다. 시그니처 기반 보조 근거도 해당 기능 404로 진단 불가를 보고하므로 최종 판단을 보류한다. 시그니처 기반 추가 근거: /vulnapp/register.jsp 요청이 404로 확인되어 약한 비밀번호 허용 여부를 진단할 수 없음.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/register.jsp가 200으로 존재한다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 대표 약한 비밀번호인 '1234', 'password', 'admin123'이 가입 성공으로 처리되지 않고 차단된 것으로 보고되어 현재 수집 범위에서는 방어된 항목으로 판단한다. 시그니처 기반 추가 근거: 대표 약한 비밀번호가 가입 성공으로 처리되지 않음. blocked=['1234', 'password', 'admin123']</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>회원가입, 비밀번호 변경, 초기화 기능에서 최소 길이, 복잡도, 사전/유출 비밀번호 차단 등 정책이 적용되는지 테스트한다. 기능 구현 후 서버 측 검증을 반드시 적용한다.</t>
+          <t>서버 측 비밀번호 정책을 유지하고 최소 길이, 복잡도, 사전 기반 취약 비밀번호 차단, 유출 비밀번호 검사 등을 지속 적용하라.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1666,19 +1666,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>수집된 인증 관련 응답은 JSESSIONID 세션 쿠키 기반이며, Authorization: Bearer 토큰이나 JWT 형식의 토큰이 응답 헤더/쿠키/본문에서 확인되지 않는다. 현재 수집 범위에서는 JWT 사용 근거가 없어 진단 대상이 아니다. 시그니처 기반 추가 근거: 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않음.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 JWT 토큰, Authorization 헤더, JWT 기반 인증 흐름 또는 토큰 변조 테스트 결과가 없고 확인된 세션 관리는 JSESSIONID 쿠키 기반이다. 시그니처 기반 보조 근거에서도 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않아 현재 JWT 미사용으로 판단한다. 시그니처 기반 추가 근거: 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않음.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>JWT를 사용하는 API가 별도로 존재한다면 alg=none, 서명 검증 우회, 만료 검증 누락 등을 추가 점검한다. 현재 확인된 세션 기반 인증에는 해당 항목이 적용되지 않는다.</t>
+          <t>현재 JWT 미사용이면 별도 조치는 불필요하다. 향후 JWT를 도입하는 경우 강력한 서명 알고리즘, alg=none 차단, 만료/issuer/audience 검증, 키 관리 정책을 적용하라.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1718,24 +1718,24 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>high</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>/vulnapp/upload.jsp는 status_code 200으로 접근 가능하고 /vulnapp/upload_process.jsp는 status_code 500 응답이 확인되지만, 실제 파일 업로드 요청, JSP 파일 업로드 성공 여부, 웹 경로에서 JSP 실행 가능 여부에 대한 수집 데이터가 없다. 시그니처 기반 보조 근거도 업로드 실행 여부가 확인되지 않았다고 보고하므로 최종 판단을 보류한다. 시그니처 기반 추가 근거: shell.jsp 업로드 시도 후 업로드 실행 여부가 확인되지 않음. upload_process.jsp 500, 저장 경로 404 등 업로드 처리 오류 또는 저장 경로 확인이 필요함.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/upload.jsp가 200이고 /vulnapp/upload_process.jsp가 500을 반환했다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 JSP 파일 업로드 후 http://15.164.60.79/vulnapp/uploads/shell.jsp 접근 시 테스트용 JSP 문자열 'JSP_UPLOAD_TEST'가 출력되어 업로드된 JSP 파일이 웹 경로에서 실행되는 것이 확인되었다. 이번 프로젝트 수동진단 기준에 따라 high로 판단한다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/uploads/shell.jsp 접근 시 테스트용 JSP 문자열 JSP_UPLOAD_TEST가 출력되어 업로드된 JSP 파일이 웹 경로에서 실행되는 것이 확인됨.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>업로드 기능에 확장자/콘텐츠 타입/매직바이트 검증, 저장 경로 실행 권한 제거, 파일명 난수화, 악성 파일 검사, 업로드 후 직접 실행 차단을 적용하고 실제 업로드 및 실행 차단 여부를 재검증한다.</t>
+          <t>JSP/JSPX/PHP 등 서버 사이드 스크립트 확장자 업로드를 차단하고, 업로드 파일은 웹 루트 외부에 저장하며 실행 권한을 제거하라. 파일명 난수화, MIME/시그니처 검증, 업로드 디렉터리의 스크립트 실행 차단 설정을 적용하라.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1770,29 +1770,29 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>/vulnapp/upload_process.jsp</t>
+          <t>/vulnapp/not_exist_4akda_404_test</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>/vulnapp/upload_process.jsp 요청이 status_code 500으로 응답했고 Tomcat 기본 오류 페이지 일부가 수집되었으나, 제공된 body_sample에는 Java 예외 클래스명, stack trace 프레임, 소스 파일/라인 번호 등 상세 스택 트레이스 노출 근거가 포함되어 있지 않다. 시그니처 기반 보조 근거도 내부 DB/예외 메시지 가능성은 언급하지만 Java/Tomcat stack trace 자체는 확인되지 않았다고 보고하여 최종 판단을 보류한다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/profile.jsp?user_idx=abc 응답에 내부 DB/예외 메시지가 노출되지만 Java/Tomcat stack trace 자체는 확인되지 않음. 원래 양호 항목으로 설계되어 사이트 수정 후 재진단 필요.</t>
+          <t>존재하지 않는 경로 /vulnapp/not_exist_4akda_404_test 요청은 404로 커스텀 오류 페이지를 반환했으며 본문에는 'Service Error', '요청을 처리하지 못했습니다', 'HTTP 404' 등 일반 안내만 포함된다. Java 예외명, 클래스명, 파일 경로, 라인 번호 등 Stack Trace는 수집된 body_sample에서 확인되지 않는다. /vulnapp/upload_process.jsp의 500 응답 샘플도 공통 HTML 레이아웃 일부만 수집되었고 스택 트레이스 노출 근거는 없다. 시그니처 기반 추가 근거: 오류 유발 요청에서 Java/Tomcat stack trace 또는 내부 예외 정보가 확인되지 않음.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>500 오류 발생 시 사용자에게는 일반화된 오류 페이지를 제공하고, 상세 예외와 스택 트레이스는 서버 로그에만 기록한다. 전체 오류 응답을 확인하여 스택 트레이스 노출 여부를 추가 점검한다.</t>
+          <t>현재처럼 사용자에게는 일반화된 오류 메시지를 제공하고 상세 예외 및 스택 트레이스는 서버 내부 로그에만 기록하라. 500 오류 페이지 전체에서도 스택 트레이스가 노출되지 않도록 전역 예외 처리를 유지하라.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SCAN-20260517-185902</t>
+          <t>SCAN-20260517-231752</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-05-17T18:59:02+09:00</t>
+          <t>2026-05-17T23:17:52+09:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1832,17 +1832,17 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>high</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에서 SSRF 점검 대상으로 볼 수 있는 /vulnapp/fetch.jsp는 status_code 404 Not Found로 응답했고, 외부 URL을 서버가 가져오는 기능이나 관련 파라미터 응답은 확인되지 않는다. 시그니처 기반 보조 근거도 /vulnapp/fetch.jsp와 내부 테스트 자원이 404로 확인되어 SSRF 진단을 수행할 수 없다고 보고하므로 최종 판단을 보류한다. 시그니처 기반 추가 근거: /vulnapp/fetch.jsp가 404로 확인되어 SSRF 진단을 수행할 수 없음. /vulnapp/internal/secret.jsp도 404라 내부 테스트 자원 확인이 필요함.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/fetch.jsp가 200으로 도달 가능하고 /vulnapp/internal/secret.jsp는 외부 직접 접근 시 403으로 차단된다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 fetch.jsp가 사용자 입력 URL을 통해 내부 URL http://127.0.0.1:8080/을 요청하고 Tomcat 내부 페이지 내용을 반환한 것으로 보고되어 SSRF로 판단한다. 시그니처 기반 추가 근거: fetch.jsp가 내부 URL http://127.0.0.1:8080/을 요청하고 Tomcat 내부 페이지 내용을 반환</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>URL fetch, webhook, 이미지 프록시 등 서버 측 요청 기능이 존재하거나 구현 예정이면 내부 IP 및 메타데이터 주소 접근 차단, 허용 목록, 리다이렉트 제한, DNS rebinding 방어를 적용하고 기능 정상화 후 재진단한다.</t>
+          <t>사용자 입력 URL을 서버가 직접 요청하는 기능은 허용 목록 기반 목적지 제한을 적용하고 localhost, 사설 IP, 링크 로컬, 메타데이터 주소 및 내부 도메인 접근을 차단하라. 리다이렉트 우회와 DNS rebinding도 고려하여 네트워크 egress 제어를 병행하라.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve webshell upload detection
</commit_message>
<xml_diff>
--- a/auto-scanner/outputs/자동진단.xlsx
+++ b/auto-scanner/outputs/자동진단.xlsx
@@ -445,7 +445,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -697,19 +697,19 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>익명 요청은 /vulnapp/admin.jsp에서 302로 /vulnapp/login.jsp로 리다이렉트되어 비로그인 접근은 차단되었으나, 일반 사용자 user1 로그인 후 동일한 관리자 페이지 요청이 200으로 응답되었고 본문에 '시스템 관리자 대시보드', 'Admin Only', '현재 서버에 가입된 모든 회원' 문구가 포함되었다. 일반 사용자 세션으로 관리자 전용 페이지 접근이 가능하므로 권한 검증 미흡으로 판단한다. 시그니처 기반 추가 근거: /vulnapp/admin.jsp 비로그인 요청은 로그인 페이지로 리다이렉트됨. 일반 사용자(user1) 로그인 세션으로 /vulnapp/admin.jsp 접근 시 200 응답과 관리자 페이지 키워드가 확인되어 관리자 권한 검증 미흡이 확인됨.</t>
+          <t>비인증 요청은 /vulnapp/admin.jsp 접근 시 302로 /vulnapp/login.jsp로 리다이렉트되었으나, 일반 사용자(user1) 로그인 후 동일 URL 요청이 status_code 200으로 응답했고 본문에 '⚙️ 시스템 관리자 대시보드', 'Admin Only', '현재 서버에 가입된 모든 회원' 문구가 포함됨. 비로그인 접근은 차단되더라도 일반 사용자 세션으로 관리자 페이지가 200 응답이므로 관리자 권한 검증 미흡으로 판단함. 시그니처 기반 추가 근거: /vulnapp/admin.jsp 비로그인 요청은 로그인 페이지로 리다이렉트됨. 일반 사용자(user1) 로그인 세션으로 /vulnapp/admin.jsp 접근 시 200 응답과 관리자 페이지 키워드가 확인되어 관리자 권한 검증 미흡이 확인됨.</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>관리자 기능은 인증 여부뿐 아니라 관리자 역할/권한을 서버 측에서 검증해야 한다. /vulnapp/admin.jsp 접근 시 세션의 role 또는 authority를 확인하고 일반 사용자는 403 또는 접근 권한 없음 페이지로 차단하라.</t>
+          <t>관리자 페이지 및 기능에 대해 서버 측 권한 검사를 적용하고, 인증 여부뿐 아니라 사용자 역할/권한이 관리자임을 확인한 뒤 접근을 허용해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -754,19 +754,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/profile.jsp?user_idx=1이 200으로 도달 가능하다는 정보만 있어 단독으로는 IDOR 여부를 확정하기 부족했으나, 시그니처 기반 보조 근거에서 profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출된 것으로 보고되었다. 시그니처 기반 추가 근거: profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출됨.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 profile.jsp?user_idx=1이 200 응답으로 접근 가능한 사실만 있어 사용자별 소유권 검증 여부를 단독 확정하기 어려웠다. 시그니처 기반 보조 근거에 따르면 profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출되어 IDOR가 확인됨. 시그니처 기반 추가 근거: profile.jsp의 user_idx 값을 변경했을 때 서로 다른 사용자 정보가 200 응답으로 노출됨.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>사용자 정보 조회 시 요청 파라미터의 user_idx만 신뢰하지 말고 세션 사용자와 조회 대상의 소유자 또는 접근 권한을 서버 측에서 검증하라. 권한 없는 객체 접근은 403으로 차단하고 식별자는 예측 가능성을 낮추는 방식을 검토하라.</t>
+          <t>사용자 정보 조회 시 세션 사용자와 조회 대상 user_idx가 일치하는지 서버 측에서 검증하고, 권한 없는 접근은 403으로 차단해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>/vulnapp/의 200 응답 헤더에는 Server, Date, Content-Type, Transfer-Encoding, Connection, Set-Cookie, Content-Encoding만 확인되며 Content-Security-Policy, X-Frame-Options, X-Content-Type-Options, Referrer-Policy, Strict-Transport-Security 등의 주요 보안 헤더가 확인되지 않는다. 시그니처 기반 추가 근거: /vulnapp/ 응답에서 주요 보안 헤더 누락: ['Content-Security-Policy', 'X-Frame-Options', 'X-Content-Type-Options', 'Referrer-Policy']</t>
+          <t>기본 페이지 응답(status_code 200) 헤더에 Server, Date, Content-Type, Transfer-Encoding, Connection, Set-Cookie, Content-Encoding만 존재하며 Content-Security-Policy, X-Frame-Options, X-Content-Type-Options, Referrer-Policy, Permissions-Policy, Strict-Transport-Security 등의 주요 보안 헤더가 확인되지 않음. 검색 페이지와 오류 페이지 응답에서도 동일하게 주요 보안 헤더가 확인되지 않음. 시그니처 기반 추가 근거: /vulnapp/ 응답에서 주요 보안 헤더 누락: ['Content-Security-Policy', 'X-Frame-Options', 'X-Content-Type-Options', 'Referrer-Policy']</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>애플리케이션 또는 nginx에서 Content-Security-Policy, X-Frame-Options 또는 frame-ancestors, X-Content-Type-Options: nosniff, Referrer-Policy 등을 설정하라. HTTPS 적용 후 HSTS도 설정하라.</t>
+          <t>CSP, X-Frame-Options 또는 frame-ancestors, X-Content-Type-Options, Referrer-Policy, Permissions-Policy를 서비스 특성에 맞게 설정하고, HTTPS 적용 후 HSTS를 설정해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -868,19 +868,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>/vulnapp/ 및 404 응답의 Server 헤더가 'nginx/1.28.3 (Ubuntu)'로 제품명, 버전, OS 정보를 노출한다. 또한 / 및 :8080/의 Tomcat 기본 페이지 본문 title/h1에 'Apache Tomcat/9.0.118' 버전이 표시된다. 시그니처 기반 추가 근거: http://15.164.60.79/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79/ body contains Apache Tomcat/; http://15.164.60.79/vulnapp/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79:8080/ body contains Apache Tomcat/</t>
+          <t>다수 응답 헤더의 Server 값이 'nginx/1.28.3 (Ubuntu)'로 노출됨. 또한 http://15.164.60.79/ 및 http://15.164.60.79:8080/ 기본 페이지 본문 title/h1에 'Apache Tomcat/9.0.118' 버전이 노출됨. 시그니처 기반 추가 근거: http://15.164.60.79/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79/ body contains Apache Tomcat/; http://15.164.60.79/vulnapp/ Server=nginx/1.28.3 (Ubuntu); http://15.164.60.79:8080/ body contains Apache Tomcat/</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>nginx server_tokens off 설정 등으로 상세 버전 노출을 제거하고, Tomcat 기본 페이지와 오류 페이지에서 제품명 및 상세 버전 정보가 노출되지 않도록 설정하라.</t>
+          <t>웹 서버 및 WAS의 버전 정보 노출을 최소화하도록 nginx server_tokens 비활성화, 프록시/애플리케이션 오류 페이지 커스터마이징, Tomcat 기본 배너 및 기본 페이지 제거를 적용해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -925,19 +925,19 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>http://15.164.60.79/ 및 http://15.164.60.79:8080/ 요청이 200으로 응답되며 본문에 '&lt;title&gt;Apache Tomcat/9.0.118&lt;/title&gt;', '&lt;h1&gt;Apache Tomcat/9.0.118&lt;/h1&gt;', 'If you're seeing this, you've successfully installed Tomcat. Congratulations!'가 포함된 Tomcat 기본 페이지가 노출된다. 시그니처 기반 추가 근거: http://15.164.60.79:8080/에서 Tomcat 기본 페이지와 Manager/Host Manager 링크 노출</t>
+          <t>http://15.164.60.79/ 및 http://15.164.60.79:8080/ 요청이 status_code 200으로 응답했고 본문에 '&lt;title&gt;Apache Tomcat/9.0.118&lt;/title&gt;', '&lt;h1&gt;Apache Tomcat/9.0.118&lt;/h1&gt;', 'If you're seeing this, you've successfully installed Tomcat. Congratulations!' 등 Tomcat 기본 설치 페이지 내용이 노출됨. 시그니처 기반 추가 근거: http://15.164.60.79:8080/에서 Tomcat 기본 페이지와 Manager/Host Manager 링크 노출</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>운영 환경에서는 Tomcat ROOT 기본 애플리케이션, docs, examples 등 기본 리소스를 제거하거나 접근을 차단하고 필요한 애플리케이션만 배포하라. 8080 포트의 외부 접근 제한도 검토하라.</t>
+          <t>운영 환경에서 Tomcat ROOT 기본 애플리케이션, docs, examples 등 기본 콘텐츠를 제거하거나 접근 제한하고, 루트 경로는 의도한 서비스 페이지 또는 404/403으로 처리해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -982,19 +982,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>/vulnapp/debug.jsp 및 /vulnapp/debug.jsp?debug=true가 200, Content-Type application/json으로 응답하며 본문에 'debug: true', db_user 'vulnuser', db_password 'vulnpass1234', api_key 'TEST-API-KEY-123456', internal_ip '10.0.0.5'가 노출된다. 이번 프로젝트 기준에 따라 medium으로 판단한다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/debug.jsp에서 debug/API 키/DB 계정/내부 IP 등 내부 정보 노출</t>
+          <t>/vulnapp/debug.jsp 및 /vulnapp/debug.jsp?debug=true 요청이 모두 status_code 200, Content-Type application/json으로 응답했고 본문에 '{ "debug": true, "db_user": "vulnuser", "db_password": "vulnpass1234", "api_key": "TEST-API-KEY-123456", "internal_ip": "10.0.0.5" }'가 포함됨. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/debug.jsp에서 debug/API 키/DB 계정/내부 IP 등 내부 정보 노출</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>운영 환경에서 debug 엔드포인트와 debug=true 기능을 비활성화하고 인증/인가를 적용하라. 노출된 DB 계정 비밀번호와 API 키는 즉시 폐기 및 재발급하라.</t>
+          <t>운영 환경에서 디버그 엔드포인트를 비활성화하거나 인증/인가로 보호하고, DB 계정, 비밀번호, API 키, 내부 IP 등 민감정보가 응답에 포함되지 않도록 제거해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1039,19 +1039,19 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 Log4j 라이브러리 사용 여부, 버전, 의존성 목록이 없었으며, 시그니처 기반 보조 근거에서도 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않았다. 현재 외부 진단 범위에서는 해당 기술 사용 증거가 없어 진단 대상 아님으로 판단한다. 시그니처 기반 추가 근거: 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않음. 서버 내부 라이브러리 확인은 수동진단으로 보완 필요.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 Log4j 라이브러리 사용 여부와 버전 정보가 없었다. 시그니처 기반 보조 근거에서도 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않아 현재 수집 범위에서는 진단 대상 아님으로 판단함. 시그니처 기반 추가 근거: 외부 HTTP 응답에서 Log4j 사용 흔적이 확인되지 않음. 서버 내부 라이브러리 확인은 수동진단으로 보완 필요.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>서버 내부 의존성 목록 또는 배포 패키지에서 Log4j 사용 여부와 버전을 주기적으로 확인하라. 향후 Log4j를 도입하거나 사용 중인 사실이 확인되면 취약 버전 여부를 점검하고 안전한 최신 버전으로 업그레이드하라.</t>
+          <t>서버의 의존성 목록, 빌드 파일, SBOM 또는 런타임 라이브러리 버전을 주기적으로 확인하고, Log4j를 사용하는 경우 보안 패치가 적용된 버전을 사용해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1096,19 +1096,19 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence의 HTML 샘플에는 /vulnapp/css/style.css 링크만 확인되고 jQuery 스크립트 경로나 버전 정보가 없었다. 시그니처 기반 보조 근거에서도 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아닌 것으로 보고되었다. 시그니처 기반 추가 근거: 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. 기본 페이지 본문 샘플에는 /vulnapp/css/style.css 링크만 확인되며 jQuery 스크립트 경로나 버전 문자열이 제공되지 않았다. 시그니처 기반 보조 근거에서도 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님으로 판단함. 시그니처 기반 추가 근거: 주요 페이지 HTML에서 jQuery 참조가 확인되지 않아 구버전 jQuery 진단 대상이 아님.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>향후 jQuery를 도입하는 경우 보안 지원되는 최신 버전을 사용하고, SCA 도구나 정적 리소스 점검으로 취약 버전 사용 여부를 주기적으로 확인하라.</t>
+          <t>향후 jQuery를 도입하거나 사용 중인 정적 리소스가 추가 확인될 경우 최신 보안 패치 버전을 사용하고 취약 버전 여부를 점검해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1153,19 +1153,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>http://15.164.60.79/는 200으로 응답하지만, https://15.164.60.79는 443 포트 연결 타임아웃으로 https_available=false이며 redirect_to_https=false로 기록되어 있다. HTTPS가 제공되지 않고 HTTP에서 HTTPS로 강제 전환되지 않아 이번 프로젝트 기준에 따라 medium으로 판단한다. 시그니처 기반 추가 근거: HTTP 접속 가능 및 HTTPS 강제 리다이렉트 미확인. https_available=False, redirect_to_https=False</t>
+          <t>HTTP 요청 http://15.164.60.79/ 은 status_code 200으로 정상 응답했으나, HTTPS 요청 https://15.164.60.79 는 'Connection to 15.164.60.79 timed out' 오류가 발생했고 https_available=false, redirect_to_https=false로 수집됨. 시그니처 기반 추가 근거: HTTP 접속 가능 및 HTTPS 강제 리다이렉트 미확인. https_available=False, redirect_to_https=False</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>유효한 TLS 인증서를 적용하여 HTTPS 서비스를 활성화하고 모든 HTTP 요청을 HTTPS로 리다이렉트하라. 로그인, 세션 쿠키, 개인정보 등 민감 정보 전송 구간은 반드시 TLS로 보호하라.</t>
+          <t>443 포트에 유효한 TLS 인증서를 적용하여 HTTPS를 제공하고, HTTP 요청은 HTTPS로 리다이렉트하며, 적용 후 HSTS를 설정해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1210,19 +1210,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>basic_page 응답의 Set-Cookie는 'JSESSIONID=...; Path=/vulnapp; HttpOnly'로 HttpOnly는 있으나 Secure 속성이 없다. SQL Injection 테스트 및 관리자 페이지 익명 요청의 JSESSIONID Set-Cookie도 Path=/vulnapp; HttpOnly만 포함하고 Secure가 없다. HTTPS가 미적용된 상태라 Secure 쿠키도 적용되지 않은 것으로 확인된다. 시그니처 기반 추가 근거: Set-Cookie=JSESSIONID=CB689639FD615B11C2C3EE1F1A8AAB44; Path=/vulnapp; HttpOnly, missing=['secure', 'samesite']</t>
+          <t>기본 페이지 응답 헤더에 'Set-Cookie: JSESSIONID=BF23AB8A677F1519152ABCE26B47CD10; Path=/vulnapp; HttpOnly'가 확인되어 HttpOnly는 설정되어 있으나 Secure 및 SameSite 속성이 없음. SQL Injection 테스트 및 관리자 페이지 비인증 요청의 Set-Cookie에서도 JSESSIONID에 Path와 HttpOnly만 확인되고 Secure/SameSite는 확인되지 않음. 시그니처 기반 추가 근거: Set-Cookie=JSESSIONID=A5D8B62B0ECD1D232677824C8436B95A; Path=/vulnapp; HttpOnly, missing=['secure', 'samesite']</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>HTTPS 적용 후 세션 쿠키에 Secure, HttpOnly, SameSite=Lax 또는 Strict 속성을 설정하라. 인증 쿠키가 평문 HTTP로 전송되지 않도록 HTTPS 강제 전환과 함께 적용하라.</t>
+          <t>세션 쿠키에 Secure, HttpOnly, SameSite=Lax 또는 Strict 속성을 설정해야 한다. Secure 속성은 HTTPS 적용과 함께 활성화해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1267,19 +1267,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>SQL Injection authentication bypass test에서 /vulnapp/login.jsp의 id 값에 조건 조작 입력을 전송한 3개 요청이 모두 302로 응답했고 Location 헤더가 http://15.164.60.79/vulnapp/admin.jsp로 설정되었다. 정상 인증 정보가 아닌 입력으로 관리자 페이지로 리다이렉트되는 반응이 확인된다. 시그니처 기반 보조 근거의 sqlmap 보조 점검에서도 인증 우회가 확인되었고, DBMS 배너는 MySQL 계열 MariaDB 11.8.6-MariaDB-5 from Ubuntu로 식별되었으며, 현재 DB 사용자는 vulnuser@localhost, 현재 데이터베이스는 vuln_db로 확인되었다. 열거된 데이터베이스는 information_schema와 vuln_db이고 현재 DB 계정은 DBA 권한은 아닌 것으로 보고되었다. 시그니처 기반 추가 근거: payload=' OR '1'='1' --, redirect_location=http://15.164.60.79/vulnapp/admin.jsp, error_based=False, auth_bypass=True, sqlmap 보조 점검 결과: DBMS 배너는 MySQL &gt;= 5.1 (MariaDB fork) / banner=11.8.6-MariaDB-5 from Ubuntu로 식별됨. DB 현재 사용자는 vulnuser@localhost로 확인됨. current database() 값은 vuln_db로 확인됨. 현재 DB 계정은 DBA 권한으로 식별되지 않음. 열거된 데이터베이스는 information_schema, vuln_db 임.</t>
+          <t>로그인 페이지에 인증 우회 페이로드를 전송한 결과, id="' OR '1'='1' -- ", pw="test" 요청이 status_code 302로 'Location: http://15.164.60.79/vulnapp/admin.jsp'를 반환함. id="admin' -- ", id="' OR 1=1 -- " 테스트도 모두 302로 /vulnapp/admin.jsp 리다이렉트됨. 일반 정상 사용자 로그인은 /vulnapp/로 리다이렉트된 반면 SQL 페이로드는 관리자 페이지로 리다이렉트되는 차이가 확인됨. 시그니처 기반 보조 근거의 sqlmap_summary에 따르면 DBMS 배너는 MySQL &gt;= 5.1 (MariaDB fork) / banner=11.8.6-MariaDB-5 from Ubuntu로 식별되었고, current_user는 vulnuser@localhost, current_db는 vuln_db로 확인되었으며, 열거된 databases는 information_schema 및 vuln_db이고 현재 DB 계정은 DBA 권한이 아닌 것으로 확인됨. 시그니처 기반 추가 근거: payload=' OR '1'='1' --, redirect_location=http://15.164.60.79/vulnapp/admin.jsp, error_based=False, auth_bypass=True, sqlmap 보조 점검 결과: DBMS 배너는 MySQL &gt;= 5.1 (MariaDB fork) / banner=11.8.6-MariaDB-5 from Ubuntu로 식별됨. DB 현재 사용자는 vulnuser@localhost로 확인됨. current database() 값은 vuln_db로 확인됨. 현재 DB 계정은 DBA 권한으로 식별되지 않음. 열거된 데이터베이스는 information_schema, vuln_db 임.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>로그인 쿼리에 Prepared Statement와 파라미터 바인딩을 사용하고 문자열 연결 방식의 SQL 생성을 제거하라. 인증 로직을 재검토하고 입력값 검증, DB 오류 메시지 비노출, 최소 권한 DB 계정 적용을 병행하라.</t>
+          <t>로그인 처리 쿼리에 Prepared Statement/파라미터 바인딩을 적용하고, 입력값 검증 및 인증 로직을 재점검해야 한다. SQL 오류 여부와 무관하게 문자열 결합 쿼리를 제거해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1324,19 +1324,19 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>/vulnapp/search.jsp의 실제 파라미터 keyword에 '&lt;script&gt;alert(1337)&lt;/script&gt;'를 전달한 응답에서 입력값이 input value 및 strong 태그 영역에 HTML 이스케이프 없이 반사되었다. 또한 '"&gt;&lt;script&gt;alert(1)&lt;/script&gt;' 입력 시 input value 속성 컨텍스트를 탈출한 스크립트 태그가 응답 본문에 포함되었다. 이번 프로젝트 기준에 따라 Reflected XSS는 medium으로 판단한다. 시그니처 기반 추가 근거: keyword 파라미터에 입력한 script 태그가 응답에 HTML escaping 없이 반영됨.</t>
+          <t>검색 페이지의 실제 파라미터 keyword에 &lt;script&gt;alert(1337)&lt;/script&gt; 요청 시 status_code 200 응답 본문에서 input value="&lt;script&gt;alert(1337)&lt;/script&gt;" 및 '&lt;strong&gt;'&lt;script&gt;alert(1337)&lt;/script&gt;'&lt;/strong&gt; 에 대한 검색 결과입니다.' 형태로 페이로드가 HTML 이스케이프 없이 반사됨. keyword='"&gt;&lt;script&gt;alert(1)&lt;/script&gt;' 요청에서도 input value=""&gt;&lt;script&gt;alert(1)&lt;/script&gt;"로 속성 탈출 가능한 형태가 확인됨. 시그니처 기반 추가 근거: keyword 파라미터에 입력한 script 태그가 응답에 HTML escaping 없이 반영됨.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>검색어 등 사용자 입력을 출력 컨텍스트에 맞게 HTML 본문, HTML 속성, JavaScript 컨텍스트별로 인코딩하라. CSP를 적용하여 스크립트 실행 위험을 완화하고 입력 검증만이 아니라 출력 인코딩을 필수로 적용하라.</t>
+          <t>출력 위치별 HTML/속성/JavaScript 컨텍스트에 맞는 인코딩을 적용하고, 사용자 입력을 그대로 HTML에 삽입하지 말아야 한다. CSP도 보조 방어로 적용해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1381,19 +1381,19 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/board.jsp가 200으로 존재한다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 /vulnapp/board.jsp에 저장한 테스트 게시글을 재조회했을 때 script 페이로드가 HTML escape된 형태로만 확인되어 Stored XSS가 차단된 것으로 보고되었다. 시그니처 기반 추가 근거: /vulnapp/board.jsp에 저장한 테스트 게시글이 재조회되었고 script 페이로드가 HTML escape된 형태로만 확인되어 Stored XSS가 차단됨.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/board.jsp가 200 응답으로 접근 가능한 사실만 있고 저장/재조회 검증 데이터가 부족했다. 시그니처 기반 보조 근거에 따르면 /vulnapp/board.jsp에 저장한 테스트 게시글이 재조회되었고 script 페이로드가 HTML escape된 형태로만 확인되어 Stored XSS가 차단됨.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>현재 게시글 출력 인코딩 정책을 유지하고, 게시글 목록/상세/댓글/프로필 등 저장 데이터가 출력되는 모든 지점에 동일한 컨텍스트 기반 이스케이프를 적용하라.</t>
+          <t>현재 출력 인코딩 정책을 유지하고, 게시글 상세/목록 및 댓글 등 모든 저장 데이터 출력 지점에 동일한 escaping 정책을 적용해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1438,19 +1438,19 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/command.jsp가 200으로 도달 가능하다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 명령어 삽입 테스트 입력에 대해 실행 결과가 노출되지 않았고 관련 페이로드가 차단된 것으로 보고되어 현재 수집 범위에서는 방어된 항목으로 판단한다. 시그니처 기반 추가 근거: /vulnapp/command.jsp 명령어 삽입 페이로드에서 실행 결과 미노출. blocked=['time_snapshot;whoami', 'host_summary&amp;&amp;id', 'uptime_check|whoami']</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/command.jsp가 200 응답으로 접근 가능한 사실만 있고 명령 실행 파라미터 및 페이로드 반응 데이터가 부족했다. 시그니처 기반 보조 근거에 따르면 command.jsp 명령어 삽입 점검에서 실행 결과가 노출되지 않았고 점검 페이로드가 차단되어 Command Injection은 확인되지 않음. 시그니처 기반 추가 근거: /vulnapp/command.jsp 명령어 삽입 페이로드에서 실행 결과 미노출. blocked=['time_snapshot;whoami', 'host_summary&amp;&amp;id', 'uptime_check|whoami']</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>작업 코드나 상태 조회 입력값은 허용 목록 기반으로 검증하고 OS 명령 문자열에 사용자 입력을 직접 결합하지 말라. 가능한 경우 OS 명령 호출 대신 안전한 서버 API를 사용하라.</t>
+          <t>작업 코드 입력값은 허용 문자만 통과시키고 OS 명령 문자열 직접 결합을 금지해야 한다. 기능 변경 시 명령 실행 경로에 대해 재검증해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1495,19 +1495,19 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>rate_limit 수집 결과에서 /vulnapp/login.jsp에 대해 10회 연속 요청을 수행했으나 blocked=false이며 각 시도는 200으로 로그인 페이지 응답을 계속 반환했다. 차단, 지연, CAPTCHA, 429 응답 등의 제한 동작이 확인되지 않았다. 시그니처 기반 추가 근거: 잘못된 비밀번호 10회 연속 요청 상태코드: [200, 200, 200, 200, 200, 200, 200, 200, 200, 200]. 제한 응답 미확인.</t>
+          <t>rate_limit 수집 결과 /vulnapp/login.jsp에 10회 로그인 시도 후 blocked=false로 기록됨. 각 시도는 status_code 200으로 동일한 로그인 페이지 형태의 응답을 반환했으며 차단, 지연, 429 응답 등의 제한 근거가 확인되지 않음. 시그니처 기반 추가 근거: 잘못된 비밀번호 10회 연속 요청 상태코드: [200, 200, 200, 200, 200, 200, 200, 200, 200, 200]. 제한 응답 미확인.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>로그인 실패 횟수에 따른 IP/계정 기반 속도 제한, 지수 백오프, CAPTCHA 또는 일시 차단 정책을 적용하고 모니터링 및 알림을 구성하라.</t>
+          <t>계정/IP/세션 단위의 로그인 시도 횟수 제한, 점진적 지연, CAPTCHA 또는 429 응답 정책을 적용하고 모니터링/알림을 구성해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1552,19 +1552,19 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>account_lockout 수집 결과에서 /vulnapp/login.jsp에 대해 10회 시도 후에도 blocked=false이고 모든 시도 응답이 200으로 계속 반환되었다. 반복 실패 후 계정 잠금 또는 일시 차단 동작이 확인되지 않았다. 시그니처 기반 추가 근거: 동일 계정 10회 실패 후에도 잠금/차단 응답 없음. statuses=[200, 200, 200, 200, 200, 200, 200, 200, 200, 200]</t>
+          <t>account_lockout 수집 결과 /vulnapp/login.jsp에 10회 시도 후 blocked=false로 기록됨. 모든 시도 응답이 status_code 200이며 계정 잠금, 잠금 안내, 인증 차단 상태를 나타내는 응답 근거가 없음. 시그니처 기반 추가 근거: 동일 계정 10회 실패 후에도 잠금/차단 응답 없음. statuses=[200, 200, 200, 200, 200, 200, 200, 200, 200, 200]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>계정별 연속 로그인 실패 횟수 기준의 일시 잠금 또는 추가 인증 절차를 적용하라. 잠금 정책은 사용자 안내와 관리자 해제 또는 자동 해제 절차를 포함해야 한다.</t>
+          <t>반복 실패 시 계정 잠금 또는 단계적 보호 정책을 적용하되, 서비스 거부 악용을 방지하기 위해 위험 기반 인증, 지연, 관리자/사용자 알림 정책을 함께 설계해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1609,19 +1609,19 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/register.jsp가 200으로 존재한다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 대표 약한 비밀번호인 '1234', 'password', 'admin123'이 가입 성공으로 처리되지 않고 차단된 것으로 보고되어 현재 수집 범위에서는 방어된 항목으로 판단한다. 시그니처 기반 추가 근거: 대표 약한 비밀번호가 가입 성공으로 처리되지 않음. blocked=['1234', 'password', 'admin123']</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/register.jsp가 200 응답으로 접근 가능한 사실만 있고 약한 비밀번호 제출 결과는 없었다. 시그니처 기반 보조 근거에 따르면 대표 약한 비밀번호 1234, password, admin123이 가입 성공으로 처리되지 않고 차단되어 약한 비밀번호 허용은 확인되지 않음. 시그니처 기반 추가 근거: 대표 약한 비밀번호가 가입 성공으로 처리되지 않음. blocked=['1234', 'password', 'admin123']</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>서버 측 비밀번호 정책을 유지하고 최소 길이, 복잡도, 사전 기반 취약 비밀번호 차단, 유출 비밀번호 검사 등을 지속 적용하라.</t>
+          <t>현재 서버 측 비밀번호 정책을 유지하고, 최소 길이, 복잡도, 사전 기반 취약 비밀번호 차단, 유출 비밀번호 차단 정책을 지속적으로 적용해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1666,19 +1666,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 JWT 토큰, Authorization 헤더, JWT 기반 인증 흐름 또는 토큰 변조 테스트 결과가 없고 확인된 세션 관리는 JSESSIONID 쿠키 기반이다. 시그니처 기반 보조 근거에서도 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않아 현재 JWT 미사용으로 판단한다. 시그니처 기반 추가 근거: 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않음.</t>
+          <t>수집된 인증 관련 응답은 JSESSIONID 세션 쿠키 기반이며, 응답 헤더나 본문에 JWT 토큰, Authorization Bearer 토큰, JWT 사용 흔적이 확인되지 않음. 따라서 현재 수집 범위에서는 JWT 검증 우회 진단 대상이 아님. 시그니처 기반 추가 근거: 로그인 응답에서 JSESSIONID 세션 쿠키만 확인되고 JWT/Bearer/access_token이 확인되지 않음.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>현재 JWT 미사용이면 별도 조치는 불필요하다. 향후 JWT를 도입하는 경우 강력한 서명 알고리즘, alg=none 차단, 만료/issuer/audience 검증, 키 관리 정책을 적용하라.</t>
+          <t>현재 수집 범위에서는 JWT 사용 근거가 없으므로 별도 조치는 불필요하다. 향후 API에서 JWT를 사용한다면 서명 검증, alg 제한, 만료 검증, 키 관리 점검이 필요하다.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1723,19 +1723,19 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/upload.jsp가 200이고 /vulnapp/upload_process.jsp가 500을 반환했다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 JSP 파일 업로드 후 http://15.164.60.79/vulnapp/uploads/shell.jsp 접근 시 테스트용 JSP 문자열 'JSP_UPLOAD_TEST'가 출력되어 업로드된 JSP 파일이 웹 경로에서 실행되는 것이 확인되었다. 이번 프로젝트 수동진단 기준에 따라 high로 판단한다. 시그니처 기반 추가 근거: http://15.164.60.79/vulnapp/uploads/shell.jsp 접근 시 테스트용 JSP 문자열 JSP_UPLOAD_TEST가 출력되어 업로드된 JSP 파일이 웹 경로에서 실행되는 것이 확인됨.</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/upload.jsp 200 응답과 /vulnapp/upload_process.jsp 500 응답만 있어 업로드 후 실행 여부를 단독 확정하기 어려웠다. 시그니처 기반 보조 근거에 따르면 업로드 응답 또는 첨부파일 링크로 확인된 http://15.164.60.79/vulnapp/fileDownload.jsp?filename=shell.jsp 접근 시 JSP_UPLOAD_TEST 문자열이 출력되어 JSP 파일 업로드 후 웹 경로에서 JSP 실행이 확인됨. 시그니처 기반 추가 근거: 게시글 목록/상세 또는 업로드 응답에서 확인된 첨부파일 링크 http://15.164.60.79/vulnapp/fileDownload.jsp?filename=shell.jsp 접근 시 JSP_UPLOAD_TEST 문자열이 출력됨. 실행 가능한 JSP 파일이 서버 디렉터리에 저장되고 외부에서 접근 가능한 URL을 통해 실행되는 것으로 확인됨. 업로드 시도: ['http://15.164.60.79/vulnapp/upload_process.jsp status=200 final_url=http://15.164.60.79/vulnapp/upload_process.jsp', 'http://15.164.60.79/vulnapp/upload.jsp status=200 final_url=http://15.164.60.79/vulnapp/upload.jsp']</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>JSP/JSPX/PHP 등 서버 사이드 스크립트 확장자 업로드를 차단하고, 업로드 파일은 웹 루트 외부에 저장하며 실행 권한을 제거하라. 파일명 난수화, MIME/시그니처 검증, 업로드 디렉터리의 스크립트 실행 차단 설정을 적용하라.</t>
+          <t>파일 업로드 시 .jsp, .jspx, .php 등 실행 가능한 확장자를 차단하고, 업로드 파일은 웹 루트 외부에 저장하며, 파일 접근은 다운로드 전용 핸들러로 처리해야 한다. 저장 디렉터리의 스크립트 실행 권한을 제거해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1780,19 +1780,19 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>존재하지 않는 경로 /vulnapp/not_exist_4akda_404_test 요청은 404로 커스텀 오류 페이지를 반환했으며 본문에는 'Service Error', '요청을 처리하지 못했습니다', 'HTTP 404' 등 일반 안내만 포함된다. Java 예외명, 클래스명, 파일 경로, 라인 번호 등 Stack Trace는 수집된 body_sample에서 확인되지 않는다. /vulnapp/upload_process.jsp의 500 응답 샘플도 공통 HTML 레이아웃 일부만 수집되었고 스택 트레이스 노출 근거는 없다. 시그니처 기반 추가 근거: 오류 유발 요청에서 Java/Tomcat stack trace 또는 내부 예외 정보가 확인되지 않음.</t>
+          <t>존재하지 않는 경로 /vulnapp/not_exist_4akda_404_test 요청은 status_code 404로 커스텀 오류 페이지를 반환했고 본문에는 '요청을 처리하지 못했습니다', 'HTTP 404' 등 일반 안내만 포함됨. Java 예외명, stack trace, 파일 경로, SQL 오류 등 상세 내부 오류 정보는 제공된 body_sample에서 확인되지 않음. /vulnapp/upload_process.jsp 500 응답은 샘플이 제한적이나 제공된 범위에서는 스택 트레이스가 확인되지 않음. 시그니처 기반 추가 근거: 오류 유발 요청에서 Java/Tomcat stack trace 또는 내부 예외 정보가 확인되지 않음.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>현재처럼 사용자에게는 일반화된 오류 메시지를 제공하고 상세 예외 및 스택 트레이스는 서버 내부 로그에만 기록하라. 500 오류 페이지 전체에서도 스택 트레이스가 노출되지 않도록 전역 예외 처리를 유지하라.</t>
+          <t>현재처럼 사용자에게는 일반화된 오류 메시지를 제공하고, 상세 예외와 스택 트레이스는 서버 내부 로그에만 기록해야 한다. 500 오류 페이지 전체에 대해서도 동일 정책을 유지해야 한다.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SCAN-20260517-231752</t>
+          <t>SCAN-20260517-234556</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-05-17T23:17:52+09:00</t>
+          <t>2026-05-17T23:45:56+09:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1837,12 +1837,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/fetch.jsp가 200으로 도달 가능하고 /vulnapp/internal/secret.jsp는 외부 직접 접근 시 403으로 차단된다는 정보만 있어 단독 판단은 어려웠다. 시그니처 기반 보조 근거에서 fetch.jsp가 사용자 입력 URL을 통해 내부 URL http://127.0.0.1:8080/을 요청하고 Tomcat 내부 페이지 내용을 반환한 것으로 보고되어 SSRF로 판단한다. 시그니처 기반 추가 근거: fetch.jsp가 내부 URL http://127.0.0.1:8080/을 요청하고 Tomcat 내부 페이지 내용을 반환</t>
+          <t>GPT 1차 판단 보류 후 시그니처 기반 결과 참고. collected_evidence에는 /vulnapp/fetch.jsp가 200 응답으로 접근 가능하고 /vulnapp/internal/secret.jsp 외부 직접 접근은 403으로 차단된 사실만 있어 SSRF 여부를 단독 확정하기 어려웠다. 시그니처 기반 보조 근거에 따르면 fetch.jsp가 내부 URL http://127.0.0.1:8080/을 요청하고 Tomcat 내부 페이지 내용을 반환하여 SSRF가 확인됨. 이는 임의 파일 읽기가 아니라 서버 측 요청 위조 문제로 판단함.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>사용자 입력 URL을 서버가 직접 요청하는 기능은 허용 목록 기반 목적지 제한을 적용하고 localhost, 사설 IP, 링크 로컬, 메타데이터 주소 및 내부 도메인 접근을 차단하라. 리다이렉트 우회와 DNS rebinding도 고려하여 네트워크 egress 제어를 병행하라.</t>
+          <t>사용자 입력 URL 요청을 제한하고 localhost, 사설 IP, 링크로컬, 클라우드 메타데이터 주소 접근을 차단해야 한다. 목적지 URL 허용 목록, DNS 리바인딩 방어, 리다이렉트 제한, 응답 필터링을 적용해야 한다.</t>
         </is>
       </c>
     </row>

</xml_diff>